<commit_message>
BSFC map got optimized
</commit_message>
<xml_diff>
--- a/НИРС2/hCVT model/BSFC.xlsx
+++ b/НИРС2/hCVT model/BSFC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Баунти\Diplom\НИРС2\hCVT model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95199C65-960F-4A29-B66A-664C5D3E6614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4856BD-8C8E-4B16-8A40-67B75310EEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="2" r:id="rId1"/>
@@ -347,7 +347,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC654685-493D-4E65-B880-F8D174A5EE76}">
-  <dimension ref="A1:C352"/>
+  <dimension ref="A1:C351"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="8.7265625" style="1"/>
@@ -355,10 +355,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1">
-        <v>1912.8205128205091</v>
+        <v>1926.4523076923001</v>
       </c>
       <c r="B1" s="1">
-        <v>100</v>
+        <v>99.450549450549403</v>
       </c>
       <c r="C1" s="1">
         <v>214</v>
@@ -366,90 +366,90 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
-        <v>1830.7692307692305</v>
+        <v>1830.76923076923</v>
       </c>
       <c r="B2" s="1">
-        <v>100</v>
+        <v>105.49450549450501</v>
       </c>
       <c r="C2" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
-        <v>1858.1196581196566</v>
+        <v>1735.0427350427301</v>
       </c>
       <c r="B3" s="1">
-        <v>102.19780219780201</v>
+        <v>91.208791208791197</v>
       </c>
       <c r="C3" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
-        <v>1899.1452991452918</v>
+        <v>2158.9743589743498</v>
       </c>
       <c r="B4" s="1">
-        <v>102.74725274725201</v>
+        <v>95.604395604395606</v>
       </c>
       <c r="C4" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
-        <v>1981.1965811965788</v>
+        <v>1570.94017094017</v>
       </c>
       <c r="B5" s="1">
-        <v>102.19780219780201</v>
+        <v>100.54945054945</v>
       </c>
       <c r="C5" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
-        <v>2063.2478632478578</v>
+        <v>1338.4615384615299</v>
       </c>
       <c r="B6" s="1">
-        <v>100</v>
+        <v>93.406593406593402</v>
       </c>
       <c r="C6" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
-        <v>2008.5470085470051</v>
+        <v>2213.6752136752102</v>
       </c>
       <c r="B7" s="1">
-        <v>97.802197802197796</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C7" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
-        <v>1912.8205128205091</v>
+        <v>2664.9572649572601</v>
       </c>
       <c r="B8" s="1">
-        <v>97.252747252747199</v>
+        <v>108.79120879120801</v>
       </c>
       <c r="C8" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
-        <v>1844.4444444444393</v>
+        <v>2459.82905982906</v>
       </c>
       <c r="B9" s="1">
-        <v>97.802197802197796</v>
+        <v>102.19780219780201</v>
       </c>
       <c r="C9" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -531,21 +531,21 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
-        <v>3553.8461538461502</v>
+        <v>1283.76068376068</v>
       </c>
       <c r="B17" s="1">
-        <v>100</v>
+        <v>102.19780219780201</v>
       </c>
       <c r="C17" s="1">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
-        <v>3512.8205128205063</v>
+        <v>3553.8461538461502</v>
       </c>
       <c r="B18" s="1">
-        <v>109.890109890109</v>
+        <v>100</v>
       </c>
       <c r="C18" s="1">
         <v>225</v>
@@ -553,10 +553,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
-        <v>3211.9658119658093</v>
+        <v>3512.8205128205063</v>
       </c>
       <c r="B19" s="1">
-        <v>115.934065934065</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C19" s="1">
         <v>225</v>
@@ -564,10 +564,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
-        <v>2801.7094017093991</v>
+        <v>3211.9658119658093</v>
       </c>
       <c r="B20" s="1">
-        <v>119.780219780219</v>
+        <v>115.934065934065</v>
       </c>
       <c r="C20" s="1">
         <v>225</v>
@@ -575,10 +575,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
-        <v>2555.5555555555547</v>
+        <v>2801.7094017093991</v>
       </c>
       <c r="B21" s="1">
-        <v>124.72527472527401</v>
+        <v>119.780219780219</v>
       </c>
       <c r="C21" s="1">
         <v>225</v>
@@ -586,10 +586,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
-        <v>2104.2735042735012</v>
+        <v>2555.5555555555547</v>
       </c>
       <c r="B22" s="1">
-        <v>119.780219780219</v>
+        <v>124.72527472527401</v>
       </c>
       <c r="C22" s="1">
         <v>225</v>
@@ -597,10 +597,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
-        <v>1707.6923076922997</v>
+        <v>2104.2735042735012</v>
       </c>
       <c r="B23" s="1">
-        <v>118.681318681318</v>
+        <v>119.780219780219</v>
       </c>
       <c r="C23" s="1">
         <v>225</v>
@@ -608,10 +608,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
-        <v>1242.7350427350432</v>
+        <v>1707.6923076922997</v>
       </c>
       <c r="B24" s="1">
-        <v>109.890109890109</v>
+        <v>118.681318681318</v>
       </c>
       <c r="C24" s="1">
         <v>225</v>
@@ -619,10 +619,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
-        <v>846.15384615384608</v>
+        <v>1242.7350427350432</v>
       </c>
       <c r="B25" s="1">
-        <v>98.351648351648294</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C25" s="1">
         <v>225</v>
@@ -630,10 +630,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
-        <v>600</v>
+        <v>846.15384615384608</v>
       </c>
       <c r="B26" s="1">
-        <v>94.505494505494497</v>
+        <v>98.351648351648294</v>
       </c>
       <c r="C26" s="1">
         <v>225</v>
@@ -641,10 +641,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
-        <v>463.24786324786385</v>
+        <v>600</v>
       </c>
       <c r="B27" s="1">
-        <v>87.912087912087898</v>
+        <v>94.505494505494497</v>
       </c>
       <c r="C27" s="1">
         <v>225</v>
@@ -652,10 +652,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
-        <v>818.80341880341905</v>
+        <v>463.24786324786385</v>
       </c>
       <c r="B28" s="1">
-        <v>80.219780219780205</v>
+        <v>87.912087912087898</v>
       </c>
       <c r="C28" s="1">
         <v>225</v>
@@ -663,10 +663,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
-        <v>1229.0598290598291</v>
+        <v>818.80341880341905</v>
       </c>
       <c r="B29" s="1">
-        <v>78.021978021978001</v>
+        <v>80.219780219780205</v>
       </c>
       <c r="C29" s="1">
         <v>225</v>
@@ -674,10 +674,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
-        <v>1475.2136752136728</v>
+        <v>1229.0598290598291</v>
       </c>
       <c r="B30" s="1">
-        <v>76.373626373626294</v>
+        <v>78.021978021978001</v>
       </c>
       <c r="C30" s="1">
         <v>225</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
-        <v>2186.3247863247798</v>
+        <v>1475.2136752136728</v>
       </c>
       <c r="B31" s="1">
-        <v>80.219780219780205</v>
+        <v>76.373626373626294</v>
       </c>
       <c r="C31" s="1">
         <v>225</v>
@@ -696,10 +696,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
-        <v>2993.1623931623917</v>
+        <v>2186.3247863247798</v>
       </c>
       <c r="B32" s="1">
-        <v>87.912087912087898</v>
+        <v>80.219780219780205</v>
       </c>
       <c r="C32" s="1">
         <v>225</v>
@@ -707,21 +707,21 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
-        <v>4100.8547008547002</v>
+        <v>2993.1623931623917</v>
       </c>
       <c r="B33" s="1">
-        <v>100</v>
+        <v>87.912087912087898</v>
       </c>
       <c r="C33" s="1">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
-        <v>3977.7777777777774</v>
+        <v>4100.8547008547002</v>
       </c>
       <c r="B34" s="1">
-        <v>109.890109890109</v>
+        <v>100</v>
       </c>
       <c r="C34" s="1">
         <v>230</v>
@@ -729,10 +729,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
-        <v>3950.4273504273428</v>
+        <v>3977.7777777777774</v>
       </c>
       <c r="B35" s="1">
-        <v>119.780219780219</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C35" s="1">
         <v>230</v>
@@ -740,10 +740,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
-        <v>3540.1709401709322</v>
+        <v>3950.4273504273428</v>
       </c>
       <c r="B36" s="1">
-        <v>129.12087912087901</v>
+        <v>119.780219780219</v>
       </c>
       <c r="C36" s="1">
         <v>230</v>
@@ -751,10 +751,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
-        <v>3006.8376068376001</v>
+        <v>3540.1709401709322</v>
       </c>
       <c r="B37" s="1">
-        <v>134.06593406593399</v>
+        <v>129.12087912087901</v>
       </c>
       <c r="C37" s="1">
         <v>230</v>
@@ -762,10 +762,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
-        <v>2788.0341880341816</v>
+        <v>3006.8376068376001</v>
       </c>
       <c r="B38" s="1">
-        <v>139.56043956043899</v>
+        <v>134.06593406593399</v>
       </c>
       <c r="C38" s="1">
         <v>230</v>
@@ -773,7 +773,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
-        <v>2569.2307692307636</v>
+        <v>2788.0341880341816</v>
       </c>
       <c r="B39" s="1">
         <v>139.56043956043899</v>
@@ -784,10 +784,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
-        <v>1694.0170940170908</v>
+        <v>2569.2307692307636</v>
       </c>
       <c r="B40" s="1">
-        <v>129.67032967032901</v>
+        <v>139.56043956043899</v>
       </c>
       <c r="C40" s="1">
         <v>230</v>
@@ -795,10 +795,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
-        <v>818.80341880341905</v>
+        <v>1694.0170940170908</v>
       </c>
       <c r="B41" s="1">
-        <v>109.890109890109</v>
+        <v>129.67032967032901</v>
       </c>
       <c r="C41" s="1">
         <v>230</v>
@@ -806,10 +806,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
-        <v>326.49572649572684</v>
+        <v>818.80341880341905</v>
       </c>
       <c r="B42" s="1">
-        <v>105.49450549450501</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C42" s="1">
         <v>230</v>
@@ -817,10 +817,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
-        <v>148.71794871794884</v>
+        <v>326.49572649572684</v>
       </c>
       <c r="B43" s="1">
-        <v>91.758241758241695</v>
+        <v>105.49450549450501</v>
       </c>
       <c r="C43" s="1">
         <v>230</v>
@@ -828,10 +828,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
-        <v>312.82051282051287</v>
+        <v>148.71794871794884</v>
       </c>
       <c r="B44" s="1">
-        <v>79.120879120879096</v>
+        <v>91.758241758241695</v>
       </c>
       <c r="C44" s="1">
         <v>230</v>
@@ -839,10 +839,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
-        <v>805.12820512820508</v>
+        <v>312.82051282051287</v>
       </c>
       <c r="B45" s="1">
-        <v>70.329670329670293</v>
+        <v>79.120879120879096</v>
       </c>
       <c r="C45" s="1">
         <v>230</v>
@@ -850,10 +850,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
-        <v>1037.6068376068372</v>
+        <v>805.12820512820508</v>
       </c>
       <c r="B46" s="1">
-        <v>69.780219780219696</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C46" s="1">
         <v>230</v>
@@ -861,10 +861,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
-        <v>1762.3931623931608</v>
+        <v>1037.6068376068372</v>
       </c>
       <c r="B47" s="1">
-        <v>70.329670329670293</v>
+        <v>69.780219780219696</v>
       </c>
       <c r="C47" s="1">
         <v>230</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
-        <v>3034.188034188026</v>
+        <v>1762.3931623931608</v>
       </c>
       <c r="B48" s="1">
-        <v>79.120879120879096</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C48" s="1">
         <v>230</v>
@@ -883,10 +883,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
-        <v>3608.547008547002</v>
+        <v>3034.188034188026</v>
       </c>
       <c r="B49" s="1">
-        <v>87.912087912087898</v>
+        <v>79.120879120879096</v>
       </c>
       <c r="C49" s="1">
         <v>230</v>
@@ -894,10 +894,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
-        <v>3868.3760683760638</v>
+        <v>3608.547008547002</v>
       </c>
       <c r="B50" s="1">
-        <v>89.560439560439505</v>
+        <v>87.912087912087898</v>
       </c>
       <c r="C50" s="1">
         <v>230</v>
@@ -905,10 +905,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
-        <v>2131.6239316239271</v>
+        <v>3868.3760683760638</v>
       </c>
       <c r="B51" s="1">
-        <v>134.06593406593399</v>
+        <v>89.560439560439505</v>
       </c>
       <c r="C51" s="1">
         <v>230</v>
@@ -916,10 +916,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
-        <v>1256.4102564102564</v>
+        <v>2131.6239316239271</v>
       </c>
       <c r="B52" s="1">
-        <v>119.780219780219</v>
+        <v>134.06593406593399</v>
       </c>
       <c r="C52" s="1">
         <v>230</v>
@@ -927,21 +927,21 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
-        <v>2788.0341880341816</v>
+        <v>1256.4102564102564</v>
       </c>
       <c r="B53" s="1">
-        <v>70.879120879120805</v>
+        <v>119.780219780219</v>
       </c>
       <c r="C53" s="1">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
-        <v>3635.8974358974283</v>
+        <v>2788.0341880341816</v>
       </c>
       <c r="B54" s="1">
-        <v>79.670329670329593</v>
+        <v>70.879120879120805</v>
       </c>
       <c r="C54" s="1">
         <v>235</v>
@@ -949,10 +949,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
-        <v>4114.5299145299086</v>
+        <v>3635.8974358974283</v>
       </c>
       <c r="B55" s="1">
-        <v>86.813186813186803</v>
+        <v>79.670329670329593</v>
       </c>
       <c r="C55" s="1">
         <v>235</v>
@@ -960,10 +960,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
-        <v>4538.4615384615354</v>
+        <v>4114.5299145299086</v>
       </c>
       <c r="B56" s="1">
-        <v>99.450549450549403</v>
+        <v>86.813186813186803</v>
       </c>
       <c r="C56" s="1">
         <v>235</v>
@@ -971,10 +971,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
-        <v>4401.7094017093959</v>
+        <v>4538.4615384615354</v>
       </c>
       <c r="B57" s="1">
-        <v>114.28571428571399</v>
+        <v>99.450549450549403</v>
       </c>
       <c r="C57" s="1">
         <v>235</v>
@@ -982,10 +982,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
-        <v>4087.1794871794823</v>
+        <v>4401.7094017093959</v>
       </c>
       <c r="B58" s="1">
-        <v>129.67032967032901</v>
+        <v>114.28571428571399</v>
       </c>
       <c r="C58" s="1">
         <v>235</v>
@@ -993,10 +993,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
-        <v>3225.6410256410181</v>
+        <v>4087.1794871794823</v>
       </c>
       <c r="B59" s="1">
-        <v>141.75824175824101</v>
+        <v>129.67032967032901</v>
       </c>
       <c r="C59" s="1">
         <v>235</v>
@@ -1004,10 +1004,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
-        <v>2829.0598290598255</v>
+        <v>3225.6410256410181</v>
       </c>
       <c r="B60" s="1">
-        <v>153.84615384615299</v>
+        <v>141.75824175824101</v>
       </c>
       <c r="C60" s="1">
         <v>235</v>
@@ -1015,7 +1015,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
-        <v>2405.1282051281978</v>
+        <v>2829.0598290598255</v>
       </c>
       <c r="B61" s="1">
         <v>153.84615384615299</v>
@@ -1026,10 +1026,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
-        <v>2104.2735042735012</v>
+        <v>2405.1282051281978</v>
       </c>
       <c r="B62" s="1">
-        <v>141.20879120879101</v>
+        <v>153.84615384615299</v>
       </c>
       <c r="C62" s="1">
         <v>235</v>
@@ -1037,10 +1037,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
-        <v>1666.6666666666647</v>
+        <v>2104.2735042735012</v>
       </c>
       <c r="B63" s="1">
-        <v>135.16483516483501</v>
+        <v>141.20879120879101</v>
       </c>
       <c r="C63" s="1">
         <v>235</v>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
-        <v>1461.5384615384614</v>
+        <v>1666.6666666666647</v>
       </c>
       <c r="B64" s="1">
-        <v>129.67032967032901</v>
+        <v>135.16483516483501</v>
       </c>
       <c r="C64" s="1">
         <v>235</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
-        <v>1037.6068376068372</v>
+        <v>1461.5384615384614</v>
       </c>
       <c r="B65" s="1">
-        <v>123.626373626373</v>
+        <v>129.67032967032901</v>
       </c>
       <c r="C65" s="1">
         <v>235</v>
@@ -1070,10 +1070,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
-        <v>818.80341880341905</v>
+        <v>1037.6068376068372</v>
       </c>
       <c r="B66" s="1">
-        <v>117.58241758241699</v>
+        <v>123.626373626373</v>
       </c>
       <c r="C66" s="1">
         <v>235</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
-        <v>545.29914529914561</v>
+        <v>818.80341880341905</v>
       </c>
       <c r="B67" s="1">
-        <v>115.384615384615</v>
+        <v>117.58241758241699</v>
       </c>
       <c r="C67" s="1">
         <v>235</v>
@@ -1092,10 +1092,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
-        <v>94.017094017094678</v>
+        <v>545.29914529914561</v>
       </c>
       <c r="B68" s="1">
-        <v>109.890109890109</v>
+        <v>115.384615384615</v>
       </c>
       <c r="C68" s="1">
         <v>235</v>
@@ -1103,10 +1103,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
-        <v>-165.81196581196536</v>
+        <v>94.017094017094678</v>
       </c>
       <c r="B69" s="1">
-        <v>100</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C69" s="1">
         <v>235</v>
@@ -1114,10 +1114,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
-        <v>-1.709401709401277</v>
+        <v>-165.81196581196536</v>
       </c>
       <c r="B70" s="1">
-        <v>79.670329670329593</v>
+        <v>100</v>
       </c>
       <c r="C70" s="1">
         <v>235</v>
@@ -1125,10 +1125,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
-        <v>340.17094017094081</v>
+        <v>-1.709401709401277</v>
       </c>
       <c r="B71" s="1">
-        <v>72.527472527472497</v>
+        <v>79.670329670329593</v>
       </c>
       <c r="C71" s="1">
         <v>235</v>
@@ -1136,10 +1136,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
-        <v>818.80341880341905</v>
+        <v>340.17094017094081</v>
       </c>
       <c r="B72" s="1">
-        <v>65.384615384615302</v>
+        <v>72.527472527472497</v>
       </c>
       <c r="C72" s="1">
         <v>235</v>
@@ -1147,10 +1147,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
-        <v>1133.3333333333333</v>
+        <v>818.80341880341905</v>
       </c>
       <c r="B73" s="1">
-        <v>65.934065934065899</v>
+        <v>65.384615384615302</v>
       </c>
       <c r="C73" s="1">
         <v>235</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
-        <v>1830.7692307692305</v>
+        <v>1133.3333333333333</v>
       </c>
       <c r="B74" s="1">
         <v>65.934065934065899</v>
@@ -1169,10 +1169,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
-        <v>2254.700854700849</v>
+        <v>1830.7692307692305</v>
       </c>
       <c r="B75" s="1">
-        <v>67.582417582417506</v>
+        <v>65.934065934065899</v>
       </c>
       <c r="C75" s="1">
         <v>235</v>
@@ -1180,10 +1180,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
-        <v>3799.9999999999941</v>
+        <v>2254.700854700849</v>
       </c>
       <c r="B76" s="1">
-        <v>136.81318681318601</v>
+        <v>67.582417582417506</v>
       </c>
       <c r="C76" s="1">
         <v>235</v>
@@ -1191,21 +1191,21 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
-        <v>3047.8632478632435</v>
+        <v>3799.9999999999941</v>
       </c>
       <c r="B77" s="1">
-        <v>67.582417582417506</v>
+        <v>136.81318681318601</v>
       </c>
       <c r="C77" s="1">
-        <v>240</v>
+        <v>235</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
-        <v>3635.8974358974283</v>
+        <v>3047.8632478632435</v>
       </c>
       <c r="B78" s="1">
-        <v>74.725274725274701</v>
+        <v>67.582417582417506</v>
       </c>
       <c r="C78" s="1">
         <v>240</v>
@@ -1213,10 +1213,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
-        <v>4210.2564102564047</v>
+        <v>3635.8974358974283</v>
       </c>
       <c r="B79" s="1">
-        <v>79.670329670329593</v>
+        <v>74.725274725274701</v>
       </c>
       <c r="C79" s="1">
         <v>240</v>
@@ -1224,10 +1224,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
-        <v>4483.7606837606836</v>
+        <v>4210.2564102564047</v>
       </c>
       <c r="B80" s="1">
-        <v>89.560439560439505</v>
+        <v>79.670329670329593</v>
       </c>
       <c r="C80" s="1">
         <v>240</v>
@@ -1235,10 +1235,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
-        <v>4743.5897435897368</v>
+        <v>4483.7606837606836</v>
       </c>
       <c r="B81" s="1">
-        <v>105.49450549450501</v>
+        <v>89.560439560439505</v>
       </c>
       <c r="C81" s="1">
         <v>240</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
-        <v>4729.9145299145284</v>
+        <v>4743.5897435897368</v>
       </c>
       <c r="B82" s="1">
-        <v>121.428571428571</v>
+        <v>105.49450549450501</v>
       </c>
       <c r="C82" s="1">
         <v>240</v>
@@ -1257,10 +1257,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
-        <v>4620.5128205128149</v>
+        <v>4729.9145299145284</v>
       </c>
       <c r="B83" s="1">
-        <v>130.21978021978001</v>
+        <v>121.428571428571</v>
       </c>
       <c r="C83" s="1">
         <v>240</v>
@@ -1268,10 +1268,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
-        <v>4210.2564102564047</v>
+        <v>4620.5128205128149</v>
       </c>
       <c r="B84" s="1">
-        <v>140.10989010988999</v>
+        <v>130.21978021978001</v>
       </c>
       <c r="C84" s="1">
         <v>240</v>
@@ -1279,10 +1279,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
-        <v>3882.0512820512813</v>
+        <v>4210.2564102564047</v>
       </c>
       <c r="B85" s="1">
-        <v>143.956043956043</v>
+        <v>140.10989010988999</v>
       </c>
       <c r="C85" s="1">
         <v>240</v>
@@ -1290,10 +1290,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
-        <v>3335.0427350427317</v>
+        <v>3882.0512820512813</v>
       </c>
       <c r="B86" s="1">
-        <v>149.450549450549</v>
+        <v>143.956043956043</v>
       </c>
       <c r="C86" s="1">
         <v>240</v>
@@ -1301,10 +1301,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
-        <v>3088.8888888888869</v>
+        <v>3335.0427350427317</v>
       </c>
       <c r="B87" s="1">
-        <v>159.34065934065899</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C87" s="1">
         <v>240</v>
@@ -1312,10 +1312,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
-        <v>2405.1282051281978</v>
+        <v>3088.8888888888869</v>
       </c>
       <c r="B88" s="1">
-        <v>162.087912087912</v>
+        <v>159.34065934065899</v>
       </c>
       <c r="C88" s="1">
         <v>240</v>
@@ -1323,10 +1323,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
-        <v>2035.8974358974313</v>
+        <v>2405.1282051281978</v>
       </c>
       <c r="B89" s="1">
-        <v>153.29670329670299</v>
+        <v>162.087912087912</v>
       </c>
       <c r="C89" s="1">
         <v>240</v>
@@ -1334,10 +1334,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
-        <v>1912.8205128205091</v>
+        <v>2035.8974358974313</v>
       </c>
       <c r="B90" s="1">
-        <v>147.25274725274701</v>
+        <v>153.29670329670299</v>
       </c>
       <c r="C90" s="1">
         <v>240</v>
@@ -1345,10 +1345,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
-        <v>1639.3162393162386</v>
+        <v>1912.8205128205091</v>
       </c>
       <c r="B91" s="1">
-        <v>144.505494505494</v>
+        <v>147.25274725274701</v>
       </c>
       <c r="C91" s="1">
         <v>240</v>
@@ -1356,10 +1356,10 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
-        <v>1119.6581196581192</v>
+        <v>1639.3162393162386</v>
       </c>
       <c r="B92" s="1">
-        <v>130.76923076923001</v>
+        <v>144.505494505494</v>
       </c>
       <c r="C92" s="1">
         <v>240</v>
@@ -1367,10 +1367,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
-        <v>613.67521367521385</v>
+        <v>1119.6581196581192</v>
       </c>
       <c r="B93" s="1">
-        <v>123.626373626373</v>
+        <v>130.76923076923001</v>
       </c>
       <c r="C93" s="1">
         <v>240</v>
@@ -1378,10 +1378,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
-        <v>-1.709401709401277</v>
+        <v>613.67521367521385</v>
       </c>
       <c r="B94" s="1">
-        <v>118.681318681318</v>
+        <v>123.626373626373</v>
       </c>
       <c r="C94" s="1">
         <v>240</v>
@@ -1389,10 +1389,10 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
-        <v>-357.26495726495125</v>
+        <v>-1.709401709401277</v>
       </c>
       <c r="B95" s="1">
-        <v>107.692307692307</v>
+        <v>118.681318681318</v>
       </c>
       <c r="C95" s="1">
         <v>240</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
-        <v>-411.96581196580371</v>
+        <v>-357.26495726495125</v>
       </c>
       <c r="B96" s="1">
-        <v>98.901098901098905</v>
+        <v>107.692307692307</v>
       </c>
       <c r="C96" s="1">
         <v>240</v>
@@ -1411,10 +1411,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
-        <v>-370.94017094016863</v>
+        <v>-411.96581196580371</v>
       </c>
       <c r="B97" s="1">
-        <v>87.912087912087898</v>
+        <v>98.901098901098905</v>
       </c>
       <c r="C97" s="1">
         <v>240</v>
@@ -1422,10 +1422,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
-        <v>-97.435897435897346</v>
+        <v>-370.94017094016863</v>
       </c>
       <c r="B98" s="1">
-        <v>74.725274725274701</v>
+        <v>87.912087912087898</v>
       </c>
       <c r="C98" s="1">
         <v>240</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
-        <v>367.52136752136789</v>
+        <v>-97.435897435897346</v>
       </c>
       <c r="B99" s="1">
-        <v>64.835164835164804</v>
+        <v>74.725274725274701</v>
       </c>
       <c r="C99" s="1">
         <v>240</v>
@@ -1444,10 +1444,10 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
-        <v>805.12820512820508</v>
+        <v>367.52136752136789</v>
       </c>
       <c r="B100" s="1">
-        <v>62.087912087912002</v>
+        <v>64.835164835164804</v>
       </c>
       <c r="C100" s="1">
         <v>240</v>
@@ -1455,7 +1455,7 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
-        <v>1037.6068376068372</v>
+        <v>805.12820512820508</v>
       </c>
       <c r="B101" s="1">
         <v>62.087912087912002</v>
@@ -1466,10 +1466,10 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
-        <v>1283.7606837606834</v>
+        <v>1037.6068376068372</v>
       </c>
       <c r="B102" s="1">
-        <v>61.538461538461497</v>
+        <v>62.087912087912002</v>
       </c>
       <c r="C102" s="1">
         <v>240</v>
@@ -1477,7 +1477,7 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
-        <v>1871.7948717948655</v>
+        <v>1283.7606837606834</v>
       </c>
       <c r="B103" s="1">
         <v>61.538461538461497</v>
@@ -1488,10 +1488,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
-        <v>2295.7264957264933</v>
+        <v>1871.7948717948655</v>
       </c>
       <c r="B104" s="1">
-        <v>63.186813186813197</v>
+        <v>61.538461538461497</v>
       </c>
       <c r="C104" s="1">
         <v>240</v>
@@ -1499,10 +1499,10 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
-        <v>2623.9316239316158</v>
+        <v>2295.7264957264933</v>
       </c>
       <c r="B105" s="1">
-        <v>64.285714285714207</v>
+        <v>63.186813186813197</v>
       </c>
       <c r="C105" s="1">
         <v>240</v>
@@ -1510,21 +1510,21 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
-        <v>4524.7863247863188</v>
+        <v>2623.9316239316158</v>
       </c>
       <c r="B106" s="1">
-        <v>77.472527472527403</v>
+        <v>64.285714285714207</v>
       </c>
       <c r="C106" s="1">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
-        <v>4798.2905982905977</v>
+        <v>4524.7863247863188</v>
       </c>
       <c r="B107" s="1">
-        <v>86.263736263736206</v>
+        <v>77.472527472527403</v>
       </c>
       <c r="C107" s="1">
         <v>245</v>
@@ -1532,10 +1532,10 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
-        <v>5085.4700854700859</v>
+        <v>4798.2905982905977</v>
       </c>
       <c r="B108" s="1">
-        <v>90.109890109890102</v>
+        <v>86.263736263736206</v>
       </c>
       <c r="C108" s="1">
         <v>245</v>
@@ -1543,10 +1543,10 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
-        <v>5181.1965811965729</v>
+        <v>5085.4700854700859</v>
       </c>
       <c r="B109" s="1">
-        <v>100</v>
+        <v>90.109890109890102</v>
       </c>
       <c r="C109" s="1">
         <v>245</v>
@@ -1554,10 +1554,10 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
-        <v>5413.6752136752084</v>
+        <v>5181.1965811965729</v>
       </c>
       <c r="B110" s="1">
-        <v>128.57142857142799</v>
+        <v>100</v>
       </c>
       <c r="C110" s="1">
         <v>245</v>
@@ -1565,10 +1565,10 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
-        <v>5495.7264957264952</v>
+        <v>5413.6752136752084</v>
       </c>
       <c r="B111" s="1">
-        <v>108.79120879120801</v>
+        <v>128.57142857142799</v>
       </c>
       <c r="C111" s="1">
         <v>245</v>
@@ -1576,10 +1576,10 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
-        <v>5290.5982905982864</v>
+        <v>5495.7264957264952</v>
       </c>
       <c r="B112" s="1">
-        <v>135.71428571428501</v>
+        <v>108.79120879120801</v>
       </c>
       <c r="C112" s="1">
         <v>245</v>
@@ -1587,10 +1587,10 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
-        <v>5112.8205128205118</v>
+        <v>5290.5982905982864</v>
       </c>
       <c r="B113" s="1">
-        <v>140.65934065933999</v>
+        <v>135.71428571428501</v>
       </c>
       <c r="C113" s="1">
         <v>245</v>
@@ -1598,10 +1598,10 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
-        <v>4948.7179487179455</v>
+        <v>4333.3333333333267</v>
       </c>
       <c r="B114" s="1">
-        <v>140.65934065933999</v>
+        <v>145.05494505494499</v>
       </c>
       <c r="C114" s="1">
         <v>245</v>
@@ -1609,10 +1609,10 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
-        <v>4333.3333333333267</v>
+        <v>3717.9487179487155</v>
       </c>
       <c r="B115" s="1">
-        <v>145.05494505494499</v>
+        <v>153.29670329670299</v>
       </c>
       <c r="C115" s="1">
         <v>245</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
-        <v>3717.9487179487155</v>
+        <v>3581.1965811965761</v>
       </c>
       <c r="B116" s="1">
-        <v>153.29670329670299</v>
+        <v>160.98901098901001</v>
       </c>
       <c r="C116" s="1">
         <v>245</v>
@@ -1631,10 +1631,10 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
-        <v>3581.1965811965761</v>
+        <v>3088.8888888888869</v>
       </c>
       <c r="B117" s="1">
-        <v>160.98901098901001</v>
+        <v>168.131868131868</v>
       </c>
       <c r="C117" s="1">
         <v>245</v>
@@ -1642,10 +1642,10 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
-        <v>3088.8888888888869</v>
+        <v>2596.5811965811899</v>
       </c>
       <c r="B118" s="1">
-        <v>168.131868131868</v>
+        <v>168.681318681318</v>
       </c>
       <c r="C118" s="1">
         <v>245</v>
@@ -1653,10 +1653,10 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
-        <v>2596.5811965811899</v>
+        <v>2076.9230769230753</v>
       </c>
       <c r="B119" s="1">
-        <v>168.681318681318</v>
+        <v>165.93406593406499</v>
       </c>
       <c r="C119" s="1">
         <v>245</v>
@@ -1664,10 +1664,10 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
-        <v>2076.9230769230753</v>
+        <v>1666.6666666666647</v>
       </c>
       <c r="B120" s="1">
-        <v>165.93406593406499</v>
+        <v>162.087912087912</v>
       </c>
       <c r="C120" s="1">
         <v>245</v>
@@ -1675,10 +1675,10 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
-        <v>1666.6666666666647</v>
+        <v>1270.0854700854693</v>
       </c>
       <c r="B121" s="1">
-        <v>162.087912087912</v>
+        <v>151.648351648351</v>
       </c>
       <c r="C121" s="1">
         <v>245</v>
@@ -1686,10 +1686,10 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
-        <v>1270.0854700854693</v>
+        <v>996.5811965811962</v>
       </c>
       <c r="B122" s="1">
-        <v>151.648351648351</v>
+        <v>146.15384615384599</v>
       </c>
       <c r="C122" s="1">
         <v>245</v>
@@ -1697,10 +1697,10 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
-        <v>996.5811965811962</v>
+        <v>627.35042735042771</v>
       </c>
       <c r="B123" s="1">
-        <v>146.15384615384599</v>
+        <v>135.16483516483501</v>
       </c>
       <c r="C123" s="1">
         <v>245</v>
@@ -1708,10 +1708,10 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
-        <v>627.35042735042771</v>
+        <v>162.39316239316275</v>
       </c>
       <c r="B124" s="1">
-        <v>135.16483516483501</v>
+        <v>128.57142857142799</v>
       </c>
       <c r="C124" s="1">
         <v>245</v>
@@ -1719,10 +1719,10 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
-        <v>162.39316239316275</v>
+        <v>-452.9914529914472</v>
       </c>
       <c r="B125" s="1">
-        <v>128.57142857142799</v>
+        <v>117.58241758241699</v>
       </c>
       <c r="C125" s="1">
         <v>245</v>
@@ -1730,10 +1730,10 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
-        <v>-452.9914529914472</v>
+        <v>-630.76923076923049</v>
       </c>
       <c r="B126" s="1">
-        <v>117.58241758241699</v>
+        <v>98.901098901098905</v>
       </c>
       <c r="C126" s="1">
         <v>245</v>
@@ -1741,10 +1741,10 @@
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
-        <v>-630.76923076923049</v>
+        <v>-548.71794871794327</v>
       </c>
       <c r="B127" s="1">
-        <v>98.901098901098905</v>
+        <v>82.967032967032907</v>
       </c>
       <c r="C127" s="1">
         <v>245</v>
@@ -1752,10 +1752,10 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
-        <v>-548.71794871794327</v>
+        <v>-220.51282051282033</v>
       </c>
       <c r="B128" s="1">
-        <v>82.967032967032907</v>
+        <v>71.428571428571402</v>
       </c>
       <c r="C128" s="1">
         <v>245</v>
@@ -1763,10 +1763,10 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
-        <v>-220.51282051282033</v>
+        <v>312.82051282051287</v>
       </c>
       <c r="B129" s="1">
-        <v>71.428571428571402</v>
+        <v>62.087912087912002</v>
       </c>
       <c r="C129" s="1">
         <v>245</v>
@@ -1774,10 +1774,10 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" s="1">
-        <v>312.82051282051287</v>
+        <v>777.77777777777806</v>
       </c>
       <c r="B130" s="1">
-        <v>62.087912087912002</v>
+        <v>58.241758241758198</v>
       </c>
       <c r="C130" s="1">
         <v>245</v>
@@ -1785,7 +1785,7 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" s="1">
-        <v>777.77777777777806</v>
+        <v>1037.6068376068372</v>
       </c>
       <c r="B131" s="1">
         <v>58.241758241758198</v>
@@ -1796,10 +1796,10 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" s="1">
-        <v>1037.6068376068372</v>
+        <v>1475.2136752136728</v>
       </c>
       <c r="B132" s="1">
-        <v>58.241758241758198</v>
+        <v>57.142857142857103</v>
       </c>
       <c r="C132" s="1">
         <v>245</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" s="1">
-        <v>1475.2136752136728</v>
+        <v>2117.9487179487187</v>
       </c>
       <c r="B133" s="1">
-        <v>57.142857142857103</v>
+        <v>58.241758241758198</v>
       </c>
       <c r="C133" s="1">
         <v>245</v>
@@ -1818,10 +1818,10 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" s="1">
-        <v>2117.9487179487187</v>
+        <v>2829.0598290598255</v>
       </c>
       <c r="B134" s="1">
-        <v>58.241758241758198</v>
+        <v>60.439560439560402</v>
       </c>
       <c r="C134" s="1">
         <v>245</v>
@@ -1829,10 +1829,10 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" s="1">
-        <v>2829.0598290598255</v>
+        <v>3198.2905982905918</v>
       </c>
       <c r="B135" s="1">
-        <v>60.439560439560402</v>
+        <v>60.989010989011</v>
       </c>
       <c r="C135" s="1">
         <v>245</v>
@@ -1840,10 +1840,10 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" s="1">
-        <v>3198.2905982905918</v>
+        <v>3690.5982905982892</v>
       </c>
       <c r="B136" s="1">
-        <v>60.989010989011</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C136" s="1">
         <v>245</v>
@@ -1851,21 +1851,21 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" s="1">
-        <v>3690.5982905982892</v>
+        <v>2705.9829059829035</v>
       </c>
       <c r="B137" s="1">
-        <v>70.329670329670293</v>
+        <v>54.945054945054899</v>
       </c>
       <c r="C137" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" s="1">
-        <v>2705.9829059829035</v>
+        <v>3280.3418803418795</v>
       </c>
       <c r="B138" s="1">
-        <v>54.945054945054899</v>
+        <v>57.142857142857103</v>
       </c>
       <c r="C138" s="1">
         <v>250</v>
@@ -1873,10 +1873,10 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" s="1">
-        <v>3280.3418803418795</v>
+        <v>4100.8547008547002</v>
       </c>
       <c r="B139" s="1">
-        <v>57.142857142857103</v>
+        <v>59.890109890109898</v>
       </c>
       <c r="C139" s="1">
         <v>250</v>
@@ -1884,10 +1884,10 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" s="1">
-        <v>4100.8547008547002</v>
+        <v>4305.9829059829008</v>
       </c>
       <c r="B140" s="1">
-        <v>59.890109890109898</v>
+        <v>69.780219780219696</v>
       </c>
       <c r="C140" s="1">
         <v>250</v>
@@ -1895,10 +1895,10 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" s="1">
-        <v>4305.9829059829008</v>
+        <v>4565.8119658119622</v>
       </c>
       <c r="B141" s="1">
-        <v>69.780219780219696</v>
+        <v>71.428571428571402</v>
       </c>
       <c r="C141" s="1">
         <v>250</v>
@@ -1906,10 +1906,10 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" s="1">
-        <v>4565.8119658119622</v>
+        <v>5099.1452991452943</v>
       </c>
       <c r="B142" s="1">
-        <v>71.428571428571402</v>
+        <v>81.868131868131798</v>
       </c>
       <c r="C142" s="1">
         <v>250</v>
@@ -1917,10 +1917,10 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143" s="1">
-        <v>5099.1452991452943</v>
+        <v>5878.6324786324712</v>
       </c>
       <c r="B143" s="1">
-        <v>81.868131868131798</v>
+        <v>91.208791208791197</v>
       </c>
       <c r="C143" s="1">
         <v>250</v>
@@ -1928,10 +1928,10 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" s="1">
-        <v>5878.6324786324712</v>
+        <v>6152.1367521367501</v>
       </c>
       <c r="B144" s="1">
-        <v>91.208791208791197</v>
+        <v>104.395604395604</v>
       </c>
       <c r="C144" s="1">
         <v>250</v>
@@ -1939,10 +1939,10 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145" s="1">
-        <v>6152.1367521367501</v>
+        <v>6138.4615384615336</v>
       </c>
       <c r="B145" s="1">
-        <v>104.395604395604</v>
+        <v>123.626373626373</v>
       </c>
       <c r="C145" s="1">
         <v>250</v>
@@ -1950,10 +1950,10 @@
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A146" s="1">
-        <v>6138.4615384615336</v>
+        <v>5851.2820512820463</v>
       </c>
       <c r="B146" s="1">
-        <v>123.626373626373</v>
+        <v>136.26373626373601</v>
       </c>
       <c r="C146" s="1">
         <v>250</v>
@@ -1961,10 +1961,10 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A147" s="1">
-        <v>5851.2820512820463</v>
+        <v>5386.3247863247834</v>
       </c>
       <c r="B147" s="1">
-        <v>136.26373626373601</v>
+        <v>143.406593406593</v>
       </c>
       <c r="C147" s="1">
         <v>250</v>
@@ -1972,10 +1972,10 @@
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A148" s="1">
-        <v>5386.3247863247834</v>
+        <v>4675.2136752136666</v>
       </c>
       <c r="B148" s="1">
-        <v>143.406593406593</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C148" s="1">
         <v>250</v>
@@ -1983,10 +1983,10 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A149" s="1">
-        <v>4675.2136752136666</v>
+        <v>4182.9059829059788</v>
       </c>
       <c r="B149" s="1">
-        <v>149.450549450549</v>
+        <v>155.49450549450501</v>
       </c>
       <c r="C149" s="1">
         <v>250</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A150" s="1">
-        <v>4182.9059829059788</v>
+        <v>3882.0512820512813</v>
       </c>
       <c r="B150" s="1">
-        <v>155.49450549450501</v>
+        <v>167.58241758241701</v>
       </c>
       <c r="C150" s="1">
         <v>250</v>
@@ -2005,10 +2005,10 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A151" s="1">
-        <v>3882.0512820512813</v>
+        <v>2952.1367521367479</v>
       </c>
       <c r="B151" s="1">
-        <v>167.58241758241701</v>
+        <v>178.57142857142799</v>
       </c>
       <c r="C151" s="1">
         <v>250</v>
@@ -2016,10 +2016,10 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A152" s="1">
-        <v>2952.1367521367479</v>
+        <v>1830.7692307692305</v>
       </c>
       <c r="B152" s="1">
-        <v>178.57142857142799</v>
+        <v>174.175824175824</v>
       </c>
       <c r="C152" s="1">
         <v>250</v>
@@ -2027,10 +2027,10 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A153" s="1">
-        <v>1830.7692307692305</v>
+        <v>1064.9572649572642</v>
       </c>
       <c r="B153" s="1">
-        <v>174.175824175824</v>
+        <v>160.98901098901001</v>
       </c>
       <c r="C153" s="1">
         <v>250</v>
@@ -2038,10 +2038,10 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A154" s="1">
-        <v>1064.9572649572642</v>
+        <v>600</v>
       </c>
       <c r="B154" s="1">
-        <v>160.98901098901001</v>
+        <v>151.098901098901</v>
       </c>
       <c r="C154" s="1">
         <v>250</v>
@@ -2049,10 +2049,10 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A155" s="1">
-        <v>600</v>
+        <v>-535.04273504273465</v>
       </c>
       <c r="B155" s="1">
-        <v>151.098901098901</v>
+        <v>132.967032967032</v>
       </c>
       <c r="C155" s="1">
         <v>250</v>
@@ -2060,10 +2060,10 @@
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A156" s="1">
-        <v>-535.04273504273465</v>
+        <v>-849.57264957264897</v>
       </c>
       <c r="B156" s="1">
-        <v>132.967032967032</v>
+        <v>111.53846153846099</v>
       </c>
       <c r="C156" s="1">
         <v>250</v>
@@ -2071,10 +2071,10 @@
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A157" s="1">
-        <v>-849.57264957264897</v>
+        <v>-740.17094017093541</v>
       </c>
       <c r="B157" s="1">
-        <v>111.53846153846099</v>
+        <v>80.219780219780205</v>
       </c>
       <c r="C157" s="1">
         <v>250</v>
@@ -2082,10 +2082,10 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158" s="1">
-        <v>-740.17094017093541</v>
+        <v>-288.88888888888141</v>
       </c>
       <c r="B158" s="1">
-        <v>80.219780219780205</v>
+        <v>66.483516483516397</v>
       </c>
       <c r="C158" s="1">
         <v>250</v>
@@ -2093,10 +2093,10 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" s="1">
-        <v>-288.88888888888141</v>
+        <v>244.4444444444448</v>
       </c>
       <c r="B159" s="1">
-        <v>66.483516483516397</v>
+        <v>57.142857142857103</v>
       </c>
       <c r="C159" s="1">
         <v>250</v>
@@ -2104,10 +2104,10 @@
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160" s="1">
-        <v>244.4444444444448</v>
+        <v>600</v>
       </c>
       <c r="B160" s="1">
-        <v>57.142857142857103</v>
+        <v>54.945054945054899</v>
       </c>
       <c r="C160" s="1">
         <v>250</v>
@@ -2115,10 +2115,10 @@
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161" s="1">
-        <v>600</v>
+        <v>1010.2564102564102</v>
       </c>
       <c r="B161" s="1">
-        <v>54.945054945054899</v>
+        <v>53.846153846153797</v>
       </c>
       <c r="C161" s="1">
         <v>250</v>
@@ -2126,10 +2126,10 @@
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162" s="1">
-        <v>1010.2564102564102</v>
+        <v>1830.7692307692305</v>
       </c>
       <c r="B162" s="1">
-        <v>53.846153846153797</v>
+        <v>52.747252747252702</v>
       </c>
       <c r="C162" s="1">
         <v>250</v>
@@ -2137,21 +2137,21 @@
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163" s="1">
-        <v>1830.7692307692305</v>
+        <v>600</v>
       </c>
       <c r="B163" s="1">
-        <v>52.747252747252702</v>
+        <v>41.758241758241702</v>
       </c>
       <c r="C163" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164" s="1">
-        <v>600</v>
+        <v>1735.0427350427346</v>
       </c>
       <c r="B164" s="1">
-        <v>41.758241758241702</v>
+        <v>42.857142857142797</v>
       </c>
       <c r="C164" s="1">
         <v>275</v>
@@ -2159,10 +2159,10 @@
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" s="1">
-        <v>1735.0427350427346</v>
+        <v>2883.7606837606777</v>
       </c>
       <c r="B165" s="1">
-        <v>42.857142857142797</v>
+        <v>44.505494505494497</v>
       </c>
       <c r="C165" s="1">
         <v>275</v>
@@ -2170,10 +2170,10 @@
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166" s="1">
-        <v>2883.7606837606777</v>
+        <v>3964.1025641025599</v>
       </c>
       <c r="B166" s="1">
-        <v>44.505494505494497</v>
+        <v>47.252747252747199</v>
       </c>
       <c r="C166" s="1">
         <v>275</v>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167" s="1">
-        <v>3964.1025641025599</v>
+        <v>4770.9401709401718</v>
       </c>
       <c r="B167" s="1">
-        <v>47.252747252747199</v>
+        <v>49.450549450549403</v>
       </c>
       <c r="C167" s="1">
         <v>275</v>
@@ -2192,10 +2192,10 @@
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A168" s="1">
-        <v>4770.9401709401718</v>
+        <v>5413.6752136752084</v>
       </c>
       <c r="B168" s="1">
-        <v>49.450549450549403</v>
+        <v>53.296703296703299</v>
       </c>
       <c r="C168" s="1">
         <v>275</v>
@@ -2203,10 +2203,10 @@
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169" s="1">
-        <v>5413.6752136752084</v>
+        <v>5851.2820512820463</v>
       </c>
       <c r="B169" s="1">
-        <v>53.296703296703299</v>
+        <v>63.186813186813197</v>
       </c>
       <c r="C169" s="1">
         <v>275</v>
@@ -2214,10 +2214,10 @@
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A170" s="1">
-        <v>5851.2820512820463</v>
+        <v>6370.9401709401682</v>
       </c>
       <c r="B170" s="1">
-        <v>63.186813186813197</v>
+        <v>74.725274725274701</v>
       </c>
       <c r="C170" s="1">
         <v>275</v>
@@ -2225,10 +2225,10 @@
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A171" s="1">
-        <v>6370.9401709401682</v>
+        <v>6685.4700854700832</v>
       </c>
       <c r="B171" s="1">
-        <v>74.725274725274701</v>
+        <v>93.956043956043899</v>
       </c>
       <c r="C171" s="1">
         <v>275</v>
@@ -2236,10 +2236,10 @@
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A172" s="1">
-        <v>6685.4700854700832</v>
+        <v>6808.5470085470051</v>
       </c>
       <c r="B172" s="1">
-        <v>93.956043956043899</v>
+        <v>120.32967032966999</v>
       </c>
       <c r="C172" s="1">
         <v>275</v>
@@ -2247,10 +2247,10 @@
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A173" s="1">
-        <v>6808.5470085470051</v>
+        <v>6589.7435897435862</v>
       </c>
       <c r="B173" s="1">
-        <v>120.32967032966999</v>
+        <v>147.25274725274701</v>
       </c>
       <c r="C173" s="1">
         <v>275</v>
@@ -2258,10 +2258,10 @@
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A174" s="1">
-        <v>6589.7435897435862</v>
+        <v>5823.9316239316186</v>
       </c>
       <c r="B174" s="1">
-        <v>147.25274725274701</v>
+        <v>164.83516483516399</v>
       </c>
       <c r="C174" s="1">
         <v>275</v>
@@ -2269,10 +2269,10 @@
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A175" s="1">
-        <v>5823.9316239316186</v>
+        <v>4948.7179487179455</v>
       </c>
       <c r="B175" s="1">
-        <v>164.83516483516399</v>
+        <v>179.12087912087901</v>
       </c>
       <c r="C175" s="1">
         <v>275</v>
@@ -2280,10 +2280,10 @@
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A176" s="1">
-        <v>4948.7179487179455</v>
+        <v>3799.9999999999941</v>
       </c>
       <c r="B176" s="1">
-        <v>179.12087912087901</v>
+        <v>192.85714285714201</v>
       </c>
       <c r="C176" s="1">
         <v>275</v>
@@ -2291,10 +2291,10 @@
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A177" s="1">
-        <v>3799.9999999999941</v>
+        <v>3225.6410256410181</v>
       </c>
       <c r="B177" s="1">
-        <v>192.85714285714201</v>
+        <v>200</v>
       </c>
       <c r="C177" s="1">
         <v>275</v>
@@ -2302,10 +2302,10 @@
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A178" s="1">
-        <v>3225.6410256410181</v>
+        <v>2514.5299145299114</v>
       </c>
       <c r="B178" s="1">
-        <v>200</v>
+        <v>198.90109890109801</v>
       </c>
       <c r="C178" s="1">
         <v>275</v>
@@ -2313,10 +2313,10 @@
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A179" s="1">
-        <v>2514.5299145299114</v>
+        <v>1830.7692307692305</v>
       </c>
       <c r="B179" s="1">
-        <v>198.90109890109801</v>
+        <v>193.406593406593</v>
       </c>
       <c r="C179" s="1">
         <v>275</v>
@@ -2324,10 +2324,10 @@
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A180" s="1">
-        <v>1830.7692307692305</v>
+        <v>736.75213675213695</v>
       </c>
       <c r="B180" s="1">
-        <v>193.406593406593</v>
+        <v>180.76923076923001</v>
       </c>
       <c r="C180" s="1">
         <v>275</v>
@@ -2335,10 +2335,10 @@
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A181" s="1">
-        <v>736.75213675213695</v>
+        <v>-247.86324786324747</v>
       </c>
       <c r="B181" s="1">
-        <v>180.76923076923001</v>
+        <v>165.93406593406499</v>
       </c>
       <c r="C181" s="1">
         <v>275</v>
@@ -2346,10 +2346,10 @@
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A182" s="1">
-        <v>-247.86324786324747</v>
+        <v>-1136.7521367521279</v>
       </c>
       <c r="B182" s="1">
-        <v>165.93406593406499</v>
+        <v>146.15384615384599</v>
       </c>
       <c r="C182" s="1">
         <v>275</v>
@@ -2357,10 +2357,10 @@
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A183" s="1">
-        <v>-1136.7521367521279</v>
+        <v>-1437.6068376068336</v>
       </c>
       <c r="B183" s="1">
-        <v>146.15384615384599</v>
+        <v>122.527472527472</v>
       </c>
       <c r="C183" s="1">
         <v>275</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A184" s="1">
-        <v>-1437.6068376068336</v>
+        <v>-1423.9316239316158</v>
       </c>
       <c r="B184" s="1">
-        <v>122.527472527472</v>
+        <v>89.560439560439505</v>
       </c>
       <c r="C184" s="1">
         <v>275</v>
@@ -2379,10 +2379,10 @@
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A185" s="1">
-        <v>-1423.9316239316158</v>
+        <v>-945.29914529914458</v>
       </c>
       <c r="B185" s="1">
-        <v>89.560439560439505</v>
+        <v>62.6373626373626</v>
       </c>
       <c r="C185" s="1">
         <v>275</v>
@@ -2390,10 +2390,10 @@
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A186" s="1">
-        <v>-945.29914529914458</v>
+        <v>-425.64102564102109</v>
       </c>
       <c r="B186" s="1">
-        <v>62.6373626373626</v>
+        <v>51.6483516483516</v>
       </c>
       <c r="C186" s="1">
         <v>275</v>
@@ -2401,10 +2401,10 @@
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A187" s="1">
-        <v>-425.64102564102109</v>
+        <v>80.34188034188071</v>
       </c>
       <c r="B187" s="1">
-        <v>51.6483516483516</v>
+        <v>43.406593406593402</v>
       </c>
       <c r="C187" s="1">
         <v>275</v>
@@ -2412,21 +2412,21 @@
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A188" s="1">
-        <v>80.34188034188071</v>
+        <v>600</v>
       </c>
       <c r="B188" s="1">
-        <v>43.406593406593402</v>
+        <v>38.461538461538403</v>
       </c>
       <c r="C188" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A189" s="1">
-        <v>600</v>
+        <v>1967.5213675213613</v>
       </c>
       <c r="B189" s="1">
-        <v>38.461538461538403</v>
+        <v>39.010989010988901</v>
       </c>
       <c r="C189" s="1">
         <v>300</v>
@@ -2434,7 +2434,7 @@
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A190" s="1">
-        <v>1967.5213675213613</v>
+        <v>3239.3162393162356</v>
       </c>
       <c r="B190" s="1">
         <v>39.010989010988901</v>
@@ -2445,10 +2445,10 @@
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A191" s="1">
-        <v>3239.3162393162356</v>
+        <v>4716.2393162393109</v>
       </c>
       <c r="B191" s="1">
-        <v>39.010989010988901</v>
+        <v>43.956043956043899</v>
       </c>
       <c r="C191" s="1">
         <v>300</v>
@@ -2456,10 +2456,10 @@
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A192" s="1">
-        <v>4716.2393162393109</v>
+        <v>5400</v>
       </c>
       <c r="B192" s="1">
-        <v>43.956043956043899</v>
+        <v>46.153846153846096</v>
       </c>
       <c r="C192" s="1">
         <v>300</v>
@@ -2467,10 +2467,10 @@
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A193" s="1">
-        <v>5400</v>
+        <v>5974.3589743589673</v>
       </c>
       <c r="B193" s="1">
-        <v>46.153846153846096</v>
+        <v>60.439560439560402</v>
       </c>
       <c r="C193" s="1">
         <v>300</v>
@@ -2478,10 +2478,10 @@
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A194" s="1">
-        <v>5974.3589743589673</v>
+        <v>6603.4188034187964</v>
       </c>
       <c r="B194" s="1">
-        <v>60.439560439560402</v>
+        <v>76.923076923076906</v>
       </c>
       <c r="C194" s="1">
         <v>300</v>
@@ -2489,10 +2489,10 @@
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A195" s="1">
-        <v>6603.4188034187964</v>
+        <v>6835.897435897431</v>
       </c>
       <c r="B195" s="1">
-        <v>76.923076923076906</v>
+        <v>90.6593406593406</v>
       </c>
       <c r="C195" s="1">
         <v>300</v>
@@ -2500,10 +2500,10 @@
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A196" s="1">
-        <v>6835.897435897431</v>
+        <v>7013.6752136752148</v>
       </c>
       <c r="B196" s="1">
-        <v>90.6593406593406</v>
+        <v>120.87912087911999</v>
       </c>
       <c r="C196" s="1">
         <v>300</v>
@@ -2511,10 +2511,10 @@
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A197" s="1">
-        <v>7013.6752136752148</v>
+        <v>6781.1965811965783</v>
       </c>
       <c r="B197" s="1">
-        <v>120.87912087911999</v>
+        <v>152.74725274725199</v>
       </c>
       <c r="C197" s="1">
         <v>300</v>
@@ -2522,10 +2522,10 @@
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A198" s="1">
-        <v>6781.1965811965783</v>
+        <v>6343.5897435897432</v>
       </c>
       <c r="B198" s="1">
-        <v>152.74725274725199</v>
+        <v>167.03296703296701</v>
       </c>
       <c r="C198" s="1">
         <v>300</v>
@@ -2533,10 +2533,10 @@
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A199" s="1">
-        <v>6343.5897435897432</v>
+        <v>6015.3846153846107</v>
       </c>
       <c r="B199" s="1">
-        <v>167.03296703296701</v>
+        <v>169.230769230769</v>
       </c>
       <c r="C199" s="1">
         <v>300</v>
@@ -2544,10 +2544,10 @@
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A200" s="1">
-        <v>6015.3846153846107</v>
+        <v>5755.5555555555484</v>
       </c>
       <c r="B200" s="1">
-        <v>169.230769230769</v>
+        <v>174.72527472527401</v>
       </c>
       <c r="C200" s="1">
         <v>300</v>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A201" s="1">
-        <v>5755.5555555555484</v>
+        <v>4770.9401709401718</v>
       </c>
       <c r="B201" s="1">
-        <v>174.72527472527401</v>
+        <v>190.10989010988999</v>
       </c>
       <c r="C201" s="1">
         <v>300</v>
@@ -2566,10 +2566,10 @@
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A202" s="1">
-        <v>4770.9401709401718</v>
+        <v>3964.1025641025599</v>
       </c>
       <c r="B202" s="1">
-        <v>190.10989010988999</v>
+        <v>200</v>
       </c>
       <c r="C202" s="1">
         <v>300</v>
@@ -2577,10 +2577,10 @@
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A203" s="1">
-        <v>3964.1025641025599</v>
+        <v>3294.0170940170879</v>
       </c>
       <c r="B203" s="1">
-        <v>200</v>
+        <v>208.79120879120799</v>
       </c>
       <c r="C203" s="1">
         <v>300</v>
@@ -2588,10 +2588,10 @@
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A204" s="1">
-        <v>3294.0170940170879</v>
+        <v>2487.1794871794846</v>
       </c>
       <c r="B204" s="1">
-        <v>208.79120879120799</v>
+        <v>208.24175824175799</v>
       </c>
       <c r="C204" s="1">
         <v>300</v>
@@ -2599,10 +2599,10 @@
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A205" s="1">
-        <v>2487.1794871794846</v>
+        <v>1694.0170940170908</v>
       </c>
       <c r="B205" s="1">
-        <v>208.24175824175799</v>
+        <v>201.648351648351</v>
       </c>
       <c r="C205" s="1">
         <v>300</v>
@@ -2610,10 +2610,10 @@
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A206" s="1">
-        <v>1694.0170940170908</v>
+        <v>791.45299145299111</v>
       </c>
       <c r="B206" s="1">
-        <v>201.648351648351</v>
+        <v>190.10989010988999</v>
       </c>
       <c r="C206" s="1">
         <v>300</v>
@@ -2621,10 +2621,10 @@
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A207" s="1">
-        <v>791.45299145299111</v>
+        <v>449.57264957264988</v>
       </c>
       <c r="B207" s="1">
-        <v>190.10989010988999</v>
+        <v>186.81318681318601</v>
       </c>
       <c r="C207" s="1">
         <v>300</v>
@@ -2632,10 +2632,10 @@
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A208" s="1">
-        <v>449.57264957264988</v>
+        <v>-439.31623931623858</v>
       </c>
       <c r="B208" s="1">
-        <v>186.81318681318601</v>
+        <v>171.97802197802099</v>
       </c>
       <c r="C208" s="1">
         <v>300</v>
@@ -2643,10 +2643,10 @@
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A209" s="1">
-        <v>-439.31623931623858</v>
+        <v>-1314.5299145299111</v>
       </c>
       <c r="B209" s="1">
-        <v>171.97802197802099</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C209" s="1">
         <v>300</v>
@@ -2654,10 +2654,10 @@
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A210" s="1">
-        <v>-1314.5299145299111</v>
+        <v>-1588.0341880341816</v>
       </c>
       <c r="B210" s="1">
-        <v>149.450549450549</v>
+        <v>126.373626373626</v>
       </c>
       <c r="C210" s="1">
         <v>300</v>
@@ -2668,7 +2668,7 @@
         <v>-1588.0341880341816</v>
       </c>
       <c r="B211" s="1">
-        <v>126.373626373626</v>
+        <v>92.307692307692193</v>
       </c>
       <c r="C211" s="1">
         <v>300</v>
@@ -2676,10 +2676,10 @@
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A212" s="1">
-        <v>-1588.0341880341816</v>
+        <v>-1423.9316239316158</v>
       </c>
       <c r="B212" s="1">
-        <v>92.307692307692193</v>
+        <v>76.923076923076906</v>
       </c>
       <c r="C212" s="1">
         <v>300</v>
@@ -2687,10 +2687,10 @@
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A213" s="1">
-        <v>-1423.9316239316158</v>
+        <v>-1068.3760683760668</v>
       </c>
       <c r="B213" s="1">
-        <v>76.923076923076906</v>
+        <v>60.989010989011</v>
       </c>
       <c r="C213" s="1">
         <v>300</v>
@@ -2698,10 +2698,10 @@
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A214" s="1">
-        <v>-1068.3760683760668</v>
+        <v>-658.11965811965661</v>
       </c>
       <c r="B214" s="1">
-        <v>60.989010989011</v>
+        <v>50.549450549450498</v>
       </c>
       <c r="C214" s="1">
         <v>300</v>
@@ -2709,10 +2709,10 @@
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A215" s="1">
-        <v>-658.11965811965661</v>
+        <v>25.641025641026658</v>
       </c>
       <c r="B215" s="1">
-        <v>50.549450549450498</v>
+        <v>39.560439560439498</v>
       </c>
       <c r="C215" s="1">
         <v>300</v>
@@ -2720,21 +2720,21 @@
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A216" s="1">
-        <v>25.641025641026658</v>
+        <v>572.64957264957263</v>
       </c>
       <c r="B216" s="1">
-        <v>39.560439560439498</v>
+        <v>30.769230769230699</v>
       </c>
       <c r="C216" s="1">
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A217" s="1">
-        <v>572.64957264957263</v>
+        <v>2528.2051282051289</v>
       </c>
       <c r="B217" s="1">
-        <v>30.769230769230699</v>
+        <v>31.3186813186813</v>
       </c>
       <c r="C217" s="1">
         <v>400</v>
@@ -2742,10 +2742,10 @@
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A218" s="1">
-        <v>2528.2051282051289</v>
+        <v>3280.3418803418795</v>
       </c>
       <c r="B218" s="1">
-        <v>31.3186813186813</v>
+        <v>31.868131868131801</v>
       </c>
       <c r="C218" s="1">
         <v>400</v>
@@ -2753,10 +2753,10 @@
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A219" s="1">
-        <v>3280.3418803418795</v>
+        <v>4511.1111111111095</v>
       </c>
       <c r="B219" s="1">
-        <v>31.868131868131801</v>
+        <v>33.516483516483497</v>
       </c>
       <c r="C219" s="1">
         <v>400</v>
@@ -2764,10 +2764,10 @@
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A220" s="1">
-        <v>4511.1111111111095</v>
+        <v>5400</v>
       </c>
       <c r="B220" s="1">
-        <v>33.516483516483497</v>
+        <v>35.164835164835097</v>
       </c>
       <c r="C220" s="1">
         <v>400</v>
@@ -2775,10 +2775,10 @@
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A221" s="1">
-        <v>5400</v>
+        <v>6070.0854700854634</v>
       </c>
       <c r="B221" s="1">
-        <v>35.164835164835097</v>
+        <v>43.956043956043899</v>
       </c>
       <c r="C221" s="1">
         <v>400</v>
@@ -2786,10 +2786,10 @@
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A222" s="1">
-        <v>6070.0854700854634</v>
+        <v>7041.0256410256407</v>
       </c>
       <c r="B222" s="1">
-        <v>43.956043956043899</v>
+        <v>76.923076923076906</v>
       </c>
       <c r="C222" s="1">
         <v>400</v>
@@ -2797,10 +2797,10 @@
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A223" s="1">
-        <v>7041.0256410256407</v>
+        <v>7410.2564102564074</v>
       </c>
       <c r="B223" s="1">
-        <v>76.923076923076906</v>
+        <v>121.428571428571</v>
       </c>
       <c r="C223" s="1">
         <v>400</v>
@@ -2808,10 +2808,10 @@
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A224" s="1">
-        <v>7410.2564102564074</v>
+        <v>6972.6495726495705</v>
       </c>
       <c r="B224" s="1">
-        <v>121.428571428571</v>
+        <v>160.43956043956001</v>
       </c>
       <c r="C224" s="1">
         <v>400</v>
@@ -2819,10 +2819,10 @@
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A225" s="1">
-        <v>6972.6495726495705</v>
+        <v>6261.5384615384546</v>
       </c>
       <c r="B225" s="1">
-        <v>160.43956043956001</v>
+        <v>180.21978021978001</v>
       </c>
       <c r="C225" s="1">
         <v>400</v>
@@ -2830,10 +2830,10 @@
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A226" s="1">
-        <v>6261.5384615384546</v>
+        <v>4866.666666666667</v>
       </c>
       <c r="B226" s="1">
-        <v>180.21978021978001</v>
+        <v>202.74725274725199</v>
       </c>
       <c r="C226" s="1">
         <v>400</v>
@@ -2841,10 +2841,10 @@
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A227" s="1">
-        <v>4866.666666666667</v>
+        <v>3430.7692307692273</v>
       </c>
       <c r="B227" s="1">
-        <v>202.74725274725199</v>
+        <v>219.780219780219</v>
       </c>
       <c r="C227" s="1">
         <v>400</v>
@@ -2852,7 +2852,7 @@
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A228" s="1">
-        <v>3430.7692307692273</v>
+        <v>2282.0512820512754</v>
       </c>
       <c r="B228" s="1">
         <v>219.780219780219</v>
@@ -2863,10 +2863,10 @@
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A229" s="1">
-        <v>2282.0512820512754</v>
+        <v>1174.3589743589741</v>
       </c>
       <c r="B229" s="1">
-        <v>219.780219780219</v>
+        <v>206.593406593406</v>
       </c>
       <c r="C229" s="1">
         <v>400</v>
@@ -2874,10 +2874,10 @@
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A230" s="1">
-        <v>1174.3589743589741</v>
+        <v>-179.48717948717933</v>
       </c>
       <c r="B230" s="1">
-        <v>206.593406593406</v>
+        <v>189.01098901098899</v>
       </c>
       <c r="C230" s="1">
         <v>400</v>
@@ -2885,10 +2885,10 @@
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A231" s="1">
-        <v>-179.48717948717933</v>
+        <v>-1068.3760683760668</v>
       </c>
       <c r="B231" s="1">
-        <v>189.01098901098899</v>
+        <v>170.32967032966999</v>
       </c>
       <c r="C231" s="1">
         <v>400</v>
@@ -2896,10 +2896,10 @@
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A232" s="1">
-        <v>-1068.3760683760668</v>
+        <v>-1683.7606837606777</v>
       </c>
       <c r="B232" s="1">
-        <v>170.32967032966999</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C232" s="1">
         <v>400</v>
@@ -2907,10 +2907,10 @@
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A233" s="1">
-        <v>-1683.7606837606777</v>
+        <v>-1847.8632478632435</v>
       </c>
       <c r="B233" s="1">
-        <v>149.450549450549</v>
+        <v>123.07692307692299</v>
       </c>
       <c r="C233" s="1">
         <v>400</v>
@@ -2918,10 +2918,10 @@
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A234" s="1">
-        <v>-1847.8632478632435</v>
+        <v>-1888.8888888888869</v>
       </c>
       <c r="B234" s="1">
-        <v>123.07692307692299</v>
+        <v>93.956043956043899</v>
       </c>
       <c r="C234" s="1">
         <v>400</v>
@@ -2929,10 +2929,10 @@
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A235" s="1">
-        <v>-1888.8888888888869</v>
+        <v>-1560.6837606837553</v>
       </c>
       <c r="B235" s="1">
-        <v>93.956043956043899</v>
+        <v>67.582417582417506</v>
       </c>
       <c r="C235" s="1">
         <v>400</v>
@@ -2940,10 +2940,10 @@
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A236" s="1">
-        <v>-1560.6837606837553</v>
+        <v>-863.24786324785759</v>
       </c>
       <c r="B236" s="1">
-        <v>67.582417582417506</v>
+        <v>42.857142857142797</v>
       </c>
       <c r="C236" s="1">
         <v>400</v>
@@ -2951,10 +2951,10 @@
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A237" s="1">
-        <v>-863.24786324785759</v>
+        <v>-1.709401709401277</v>
       </c>
       <c r="B237" s="1">
-        <v>42.857142857142797</v>
+        <v>31.3186813186813</v>
       </c>
       <c r="C237" s="1">
         <v>400</v>
@@ -2962,18 +2962,18 @@
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A238" s="1">
-        <v>-1.709401709401277</v>
+        <v>586.32478632478694</v>
       </c>
       <c r="B238" s="1">
-        <v>31.3186813186813</v>
+        <v>25.274725274725199</v>
       </c>
       <c r="C238" s="1">
-        <v>400</v>
+        <v>500</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A239" s="1">
-        <v>586.32478632478694</v>
+        <v>2022.2222222222226</v>
       </c>
       <c r="B239" s="1">
         <v>25.274725274725199</v>
@@ -2984,10 +2984,10 @@
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A240" s="1">
-        <v>2022.2222222222226</v>
+        <v>3225.6410256410181</v>
       </c>
       <c r="B240" s="1">
-        <v>25.274725274725199</v>
+        <v>25.8241758241758</v>
       </c>
       <c r="C240" s="1">
         <v>500</v>
@@ -2995,10 +2995,10 @@
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A241" s="1">
-        <v>3225.6410256410181</v>
+        <v>5386.3247863247834</v>
       </c>
       <c r="B241" s="1">
-        <v>25.8241758241758</v>
+        <v>27.4725274725274</v>
       </c>
       <c r="C241" s="1">
         <v>500</v>
@@ -3006,10 +3006,10 @@
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A242" s="1">
-        <v>5386.3247863247834</v>
+        <v>5960.6837606837589</v>
       </c>
       <c r="B242" s="1">
-        <v>27.4725274725274</v>
+        <v>29.6703296703296</v>
       </c>
       <c r="C242" s="1">
         <v>500</v>
@@ -3017,10 +3017,10 @@
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A243" s="1">
-        <v>5960.6837606837589</v>
+        <v>7109.4017094017099</v>
       </c>
       <c r="B243" s="1">
-        <v>29.6703296703296</v>
+        <v>62.087912087912002</v>
       </c>
       <c r="C243" s="1">
         <v>500</v>
@@ -3028,10 +3028,10 @@
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A244" s="1">
-        <v>7109.4017094017099</v>
+        <v>7547.0085470085478</v>
       </c>
       <c r="B244" s="1">
-        <v>62.087912087912002</v>
+        <v>96.703296703296701</v>
       </c>
       <c r="C244" s="1">
         <v>500</v>
@@ -3039,10 +3039,10 @@
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A245" s="1">
-        <v>7547.0085470085478</v>
+        <v>7683.7606837606781</v>
       </c>
       <c r="B245" s="1">
-        <v>96.703296703296701</v>
+        <v>124.72527472527401</v>
       </c>
       <c r="C245" s="1">
         <v>500</v>
@@ -3050,10 +3050,10 @@
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A246" s="1">
-        <v>7683.7606837606781</v>
+        <v>7437.6068376068333</v>
       </c>
       <c r="B246" s="1">
-        <v>124.72527472527401</v>
+        <v>152.74725274725199</v>
       </c>
       <c r="C246" s="1">
         <v>500</v>
@@ -3061,10 +3061,10 @@
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A247" s="1">
-        <v>7437.6068376068333</v>
+        <v>6917.9487179487178</v>
       </c>
       <c r="B247" s="1">
-        <v>152.74725274725199</v>
+        <v>179.12087912087901</v>
       </c>
       <c r="C247" s="1">
         <v>500</v>
@@ -3072,10 +3072,10 @@
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A248" s="1">
-        <v>6917.9487179487178</v>
+        <v>6152.1367521367501</v>
       </c>
       <c r="B248" s="1">
-        <v>179.12087912087901</v>
+        <v>197.25274725274701</v>
       </c>
       <c r="C248" s="1">
         <v>500</v>
@@ -3083,10 +3083,10 @@
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A249" s="1">
-        <v>6152.1367521367501</v>
+        <v>4962.3931623931549</v>
       </c>
       <c r="B249" s="1">
-        <v>197.25274725274701</v>
+        <v>215.38461538461499</v>
       </c>
       <c r="C249" s="1">
         <v>500</v>
@@ -3094,10 +3094,10 @@
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A250" s="1">
-        <v>4962.3931623931549</v>
+        <v>3895.7264957264902</v>
       </c>
       <c r="B250" s="1">
-        <v>215.38461538461499</v>
+        <v>225.274725274725</v>
       </c>
       <c r="C250" s="1">
         <v>500</v>
@@ -3105,10 +3105,10 @@
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A251" s="1">
-        <v>3895.7264957264902</v>
+        <v>2678.6324786324772</v>
       </c>
       <c r="B251" s="1">
-        <v>225.274725274725</v>
+        <v>229.67032967032901</v>
       </c>
       <c r="C251" s="1">
         <v>500</v>
@@ -3116,10 +3116,10 @@
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A252" s="1">
-        <v>2678.6324786324772</v>
+        <v>1598.290598290595</v>
       </c>
       <c r="B252" s="1">
-        <v>229.67032967032901</v>
+        <v>219.780219780219</v>
       </c>
       <c r="C252" s="1">
         <v>500</v>
@@ -3127,10 +3127,10 @@
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A253" s="1">
-        <v>1598.290598290595</v>
+        <v>-398.29059829059486</v>
       </c>
       <c r="B253" s="1">
-        <v>219.780219780219</v>
+        <v>201.098901098901</v>
       </c>
       <c r="C253" s="1">
         <v>500</v>
@@ -3138,10 +3138,10 @@
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A254" s="1">
-        <v>-398.29059829059486</v>
+        <v>-1478.6324786324772</v>
       </c>
       <c r="B254" s="1">
-        <v>201.098901098901</v>
+        <v>172.52747252747201</v>
       </c>
       <c r="C254" s="1">
         <v>500</v>
@@ -3149,10 +3149,10 @@
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A255" s="1">
-        <v>-1478.6324786324772</v>
+        <v>-2217.0940170940103</v>
       </c>
       <c r="B255" s="1">
-        <v>172.52747252747201</v>
+        <v>139.56043956043899</v>
       </c>
       <c r="C255" s="1">
         <v>500</v>
@@ -3160,10 +3160,10 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A256" s="1">
-        <v>-2217.0940170940103</v>
+        <v>-2271.7948717948716</v>
       </c>
       <c r="B256" s="1">
-        <v>139.56043956043899</v>
+        <v>97.802197802197796</v>
       </c>
       <c r="C256" s="1">
         <v>500</v>
@@ -3171,10 +3171,10 @@
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A257" s="1">
-        <v>-2271.7948717948716</v>
+        <v>-2011.9658119658093</v>
       </c>
       <c r="B257" s="1">
-        <v>97.802197802197796</v>
+        <v>71.428571428571402</v>
       </c>
       <c r="C257" s="1">
         <v>500</v>
@@ -3182,32 +3182,32 @@
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A258" s="1">
-        <v>-2011.9658119658093</v>
+        <v>-1464.9572649572597</v>
       </c>
       <c r="B258" s="1">
-        <v>71.428571428571402</v>
+        <v>45.054945054945001</v>
       </c>
       <c r="C258" s="1">
         <v>500</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A259" s="1">
-        <v>-1464.9572649572597</v>
+        <v>-740.17094017093541</v>
       </c>
       <c r="B259" s="1">
-        <v>45.054945054945001</v>
+        <v>30.769230769230699</v>
       </c>
       <c r="C259" s="1">
         <v>500</v>
       </c>
     </row>
-    <row r="260" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A260" s="1">
-        <v>-740.17094017093541</v>
+        <v>189.74358974359069</v>
       </c>
       <c r="B260" s="1">
-        <v>30.769230769230699</v>
+        <v>24.1758241758242</v>
       </c>
       <c r="C260" s="1">
         <v>500</v>
@@ -3215,18 +3215,18 @@
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A261" s="1">
-        <v>189.74358974359069</v>
+        <v>600</v>
       </c>
       <c r="B261" s="1">
-        <v>24.1758241758242</v>
+        <v>19.230769230769202</v>
       </c>
       <c r="C261" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A262" s="1">
-        <v>600</v>
+        <v>1967.5213675213613</v>
       </c>
       <c r="B262" s="1">
         <v>19.230769230769202</v>
@@ -3237,10 +3237,10 @@
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A263" s="1">
-        <v>1967.5213675213613</v>
+        <v>3252.9914529914445</v>
       </c>
       <c r="B263" s="1">
-        <v>19.230769230769202</v>
+        <v>20.879120879120901</v>
       </c>
       <c r="C263" s="1">
         <v>600</v>
@@ -3248,10 +3248,10 @@
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A264" s="1">
-        <v>3252.9914529914445</v>
+        <v>5400</v>
       </c>
       <c r="B264" s="1">
-        <v>20.879120879120901</v>
+        <v>21.9780219780219</v>
       </c>
       <c r="C264" s="1">
         <v>600</v>
@@ -3259,10 +3259,10 @@
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A265" s="1">
-        <v>5400</v>
+        <v>6124.7863247863243</v>
       </c>
       <c r="B265" s="1">
-        <v>21.9780219780219</v>
+        <v>25.274725274725199</v>
       </c>
       <c r="C265" s="1">
         <v>600</v>
@@ -3270,10 +3270,10 @@
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A266" s="1">
-        <v>6124.7863247863243</v>
+        <v>7013.6752136752148</v>
       </c>
       <c r="B266" s="1">
-        <v>25.274725274725199</v>
+        <v>47.802197802197803</v>
       </c>
       <c r="C266" s="1">
         <v>600</v>
@@ -3281,10 +3281,10 @@
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A267" s="1">
-        <v>7013.6752136752148</v>
+        <v>7738.461538461539</v>
       </c>
       <c r="B267" s="1">
-        <v>47.802197802197803</v>
+        <v>101.648351648351</v>
       </c>
       <c r="C267" s="1">
         <v>600</v>
@@ -3292,10 +3292,10 @@
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A268" s="1">
-        <v>7738.461538461539</v>
+        <v>7820.5128205128176</v>
       </c>
       <c r="B268" s="1">
-        <v>101.648351648351</v>
+        <v>127.47252747252701</v>
       </c>
       <c r="C268" s="1">
         <v>600</v>
@@ -3303,10 +3303,10 @@
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A269" s="1">
-        <v>7820.5128205128176</v>
+        <v>7519.6581196581201</v>
       </c>
       <c r="B269" s="1">
-        <v>127.47252747252701</v>
+        <v>157.142857142857</v>
       </c>
       <c r="C269" s="1">
         <v>600</v>
@@ -3314,10 +3314,10 @@
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A270" s="1">
-        <v>7519.6581196581201</v>
+        <v>7382.9059829059806</v>
       </c>
       <c r="B270" s="1">
-        <v>157.142857142857</v>
+        <v>172.52747252747201</v>
       </c>
       <c r="C270" s="1">
         <v>600</v>
@@ -3325,10 +3325,10 @@
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A271" s="1">
-        <v>7382.9059829059806</v>
+        <v>6589.7435897435862</v>
       </c>
       <c r="B271" s="1">
-        <v>172.52747252747201</v>
+        <v>196.70329670329599</v>
       </c>
       <c r="C271" s="1">
         <v>600</v>
@@ -3336,10 +3336,10 @@
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A272" s="1">
-        <v>6589.7435897435862</v>
+        <v>5714.5299145299141</v>
       </c>
       <c r="B272" s="1">
-        <v>196.70329670329599</v>
+        <v>215.38461538461499</v>
       </c>
       <c r="C272" s="1">
         <v>600</v>
@@ -3347,10 +3347,10 @@
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A273" s="1">
-        <v>5714.5299145299141</v>
+        <v>4729.9145299145284</v>
       </c>
       <c r="B273" s="1">
-        <v>215.38461538461499</v>
+        <v>227.47252747252699</v>
       </c>
       <c r="C273" s="1">
         <v>600</v>
@@ -3358,10 +3358,10 @@
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A274" s="1">
-        <v>4729.9145299145284</v>
+        <v>3649.5726495726458</v>
       </c>
       <c r="B274" s="1">
-        <v>227.47252747252699</v>
+        <v>236.26373626373601</v>
       </c>
       <c r="C274" s="1">
         <v>600</v>
@@ -3369,10 +3369,10 @@
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A275" s="1">
-        <v>3649.5726495726458</v>
+        <v>2801.7094017093991</v>
       </c>
       <c r="B275" s="1">
-        <v>236.26373626373601</v>
+        <v>238.461538461538</v>
       </c>
       <c r="C275" s="1">
         <v>600</v>
@@ -3380,10 +3380,10 @@
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A276" s="1">
-        <v>2801.7094017093991</v>
+        <v>2213.6752136752057</v>
       </c>
       <c r="B276" s="1">
-        <v>238.461538461538</v>
+        <v>237.912087912087</v>
       </c>
       <c r="C276" s="1">
         <v>600</v>
@@ -3391,10 +3391,10 @@
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A277" s="1">
-        <v>2213.6752136752057</v>
+        <v>1174.3589743589741</v>
       </c>
       <c r="B277" s="1">
-        <v>237.912087912087</v>
+        <v>224.72527472527401</v>
       </c>
       <c r="C277" s="1">
         <v>600</v>
@@ -3402,10 +3402,10 @@
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A278" s="1">
-        <v>1174.3589743589741</v>
+        <v>-193.16239316239239</v>
       </c>
       <c r="B278" s="1">
-        <v>224.72527472527401</v>
+        <v>212.087912087912</v>
       </c>
       <c r="C278" s="1">
         <v>600</v>
@@ -3413,10 +3413,10 @@
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A279" s="1">
-        <v>-193.16239316239239</v>
+        <v>-1232.4786324786241</v>
       </c>
       <c r="B279" s="1">
-        <v>212.087912087912</v>
+        <v>190.65934065933999</v>
       </c>
       <c r="C279" s="1">
         <v>600</v>
@@ -3424,10 +3424,10 @@
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A280" s="1">
-        <v>-1232.4786324786241</v>
+        <v>-2025.6410256410181</v>
       </c>
       <c r="B280" s="1">
-        <v>190.65934065933999</v>
+        <v>167.03296703296701</v>
       </c>
       <c r="C280" s="1">
         <v>600</v>
@@ -3435,10 +3435,10 @@
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A281" s="1">
-        <v>-2025.6410256410181</v>
+        <v>-2435.8974358974283</v>
       </c>
       <c r="B281" s="1">
-        <v>167.03296703296701</v>
+        <v>139.01098901098899</v>
       </c>
       <c r="C281" s="1">
         <v>600</v>
@@ -3446,10 +3446,10 @@
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A282" s="1">
-        <v>-2435.8974358974283</v>
+        <v>-2545.2991452991419</v>
       </c>
       <c r="B282" s="1">
-        <v>139.01098901098899</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C282" s="1">
         <v>600</v>
@@ -3457,10 +3457,10 @@
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A283" s="1">
-        <v>-2545.2991452991419</v>
+        <v>-2381.1965811965761</v>
       </c>
       <c r="B283" s="1">
-        <v>109.890109890109</v>
+        <v>84.615384615384599</v>
       </c>
       <c r="C283" s="1">
         <v>600</v>
@@ -3468,10 +3468,10 @@
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A284" s="1">
-        <v>-2381.1965811965761</v>
+        <v>-1957.264957264957</v>
       </c>
       <c r="B284" s="1">
-        <v>84.615384615384599</v>
+        <v>56.593406593406598</v>
       </c>
       <c r="C284" s="1">
         <v>600</v>
@@ -3479,10 +3479,10 @@
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A285" s="1">
-        <v>-1957.264957264957</v>
+        <v>-1492.307692307686</v>
       </c>
       <c r="B285" s="1">
-        <v>56.593406593406598</v>
+        <v>38.461538461538403</v>
       </c>
       <c r="C285" s="1">
         <v>600</v>
@@ -3490,10 +3490,10 @@
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A286" s="1">
-        <v>-1492.307692307686</v>
+        <v>-781.19658119657879</v>
       </c>
       <c r="B286" s="1">
-        <v>38.461538461538403</v>
+        <v>24.1758241758242</v>
       </c>
       <c r="C286" s="1">
         <v>600</v>
@@ -3501,10 +3501,10 @@
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A287" s="1">
-        <v>-781.19658119657879</v>
+        <v>-206.83760683760647</v>
       </c>
       <c r="B287" s="1">
-        <v>24.1758241758242</v>
+        <v>19.230769230769202</v>
       </c>
       <c r="C287" s="1">
         <v>600</v>
@@ -3512,21 +3512,21 @@
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A288" s="1">
-        <v>-206.83760683760647</v>
+        <v>613.67521367521385</v>
       </c>
       <c r="B288" s="1">
-        <v>19.230769230769202</v>
+        <v>9.3406593406593199</v>
       </c>
       <c r="C288" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A289" s="1">
-        <v>613.67521367521385</v>
+        <v>1270.0854700854693</v>
       </c>
       <c r="B289" s="1">
-        <v>9.3406593406593199</v>
+        <v>9.8901098901098905</v>
       </c>
       <c r="C289" s="1">
         <v>700</v>
@@ -3534,10 +3534,10 @@
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A290" s="1">
-        <v>1270.0854700854693</v>
+        <v>1434.1880341880344</v>
       </c>
       <c r="B290" s="1">
-        <v>9.8901098901098905</v>
+        <v>7.6923076923076703</v>
       </c>
       <c r="C290" s="1">
         <v>700</v>
@@ -3545,10 +3545,10 @@
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A291" s="1">
-        <v>1434.1880341880344</v>
+        <v>1844.4444444444393</v>
       </c>
       <c r="B291" s="1">
-        <v>7.6923076923076703</v>
+        <v>8.7912087912088097</v>
       </c>
       <c r="C291" s="1">
         <v>700</v>
@@ -3556,10 +3556,10 @@
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A292" s="1">
-        <v>1844.4444444444393</v>
+        <v>2637.6068376068333</v>
       </c>
       <c r="B292" s="1">
-        <v>8.7912087912088097</v>
+        <v>9.8901098901098905</v>
       </c>
       <c r="C292" s="1">
         <v>700</v>
@@ -3567,7 +3567,7 @@
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A293" s="1">
-        <v>2637.6068376068333</v>
+        <v>3266.6666666666615</v>
       </c>
       <c r="B293" s="1">
         <v>9.8901098901098905</v>
@@ -3578,10 +3578,10 @@
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A294" s="1">
-        <v>3266.6666666666615</v>
+        <v>5263.2478632478606</v>
       </c>
       <c r="B294" s="1">
-        <v>9.8901098901098905</v>
+        <v>10.439560439560401</v>
       </c>
       <c r="C294" s="1">
         <v>700</v>
@@ -3589,10 +3589,10 @@
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A295" s="1">
-        <v>5263.2478632478606</v>
+        <v>5427.3504273504259</v>
       </c>
       <c r="B295" s="1">
-        <v>10.439560439560401</v>
+        <v>8.7912087912088097</v>
       </c>
       <c r="C295" s="1">
         <v>700</v>
@@ -3600,10 +3600,10 @@
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A296" s="1">
-        <v>5427.3504273504259</v>
+        <v>5687.1794871794882</v>
       </c>
       <c r="B296" s="1">
-        <v>8.7912087912088097</v>
+        <v>13.186813186813101</v>
       </c>
       <c r="C296" s="1">
         <v>700</v>
@@ -3611,10 +3611,10 @@
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A297" s="1">
-        <v>5687.1794871794882</v>
+        <v>6917.9487179487178</v>
       </c>
       <c r="B297" s="1">
-        <v>13.186813186813101</v>
+        <v>28.571428571428498</v>
       </c>
       <c r="C297" s="1">
         <v>700</v>
@@ -3622,10 +3622,10 @@
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A298" s="1">
-        <v>6917.9487179487178</v>
+        <v>7806.8376068376092</v>
       </c>
       <c r="B298" s="1">
-        <v>28.571428571428498</v>
+        <v>68.131868131868103</v>
       </c>
       <c r="C298" s="1">
         <v>700</v>
@@ -3633,10 +3633,10 @@
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A299" s="1">
-        <v>7806.8376068376092</v>
+        <v>8094.0170940170865</v>
       </c>
       <c r="B299" s="1">
-        <v>68.131868131868103</v>
+        <v>101.098901098901</v>
       </c>
       <c r="C299" s="1">
         <v>700</v>
@@ -3644,10 +3644,10 @@
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A300" s="1">
-        <v>8094.0170940170865</v>
+        <v>8176.0683760683751</v>
       </c>
       <c r="B300" s="1">
-        <v>101.098901098901</v>
+        <v>125.274725274725</v>
       </c>
       <c r="C300" s="1">
         <v>700</v>
@@ -3655,10 +3655,10 @@
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A301" s="1">
-        <v>8176.0683760683751</v>
+        <v>7984.615384615382</v>
       </c>
       <c r="B301" s="1">
-        <v>125.274725274725</v>
+        <v>150.54945054945</v>
       </c>
       <c r="C301" s="1">
         <v>700</v>
@@ -3666,10 +3666,10 @@
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A302" s="1">
-        <v>7984.615384615382</v>
+        <v>7875.2136752136694</v>
       </c>
       <c r="B302" s="1">
-        <v>150.54945054945</v>
+        <v>168.681318681318</v>
       </c>
       <c r="C302" s="1">
         <v>700</v>
@@ -3677,10 +3677,10 @@
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A303" s="1">
-        <v>7875.2136752136694</v>
+        <v>7246.1538461538412</v>
       </c>
       <c r="B303" s="1">
-        <v>168.681318681318</v>
+        <v>192.85714285714201</v>
       </c>
       <c r="C303" s="1">
         <v>700</v>
@@ -3688,10 +3688,10 @@
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A304" s="1">
-        <v>7246.1538461538412</v>
+        <v>6562.3931623931603</v>
       </c>
       <c r="B304" s="1">
-        <v>192.85714285714201</v>
+        <v>208.24175824175799</v>
       </c>
       <c r="C304" s="1">
         <v>700</v>
@@ -3699,10 +3699,10 @@
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A305" s="1">
-        <v>6562.3931623931603</v>
+        <v>5577.7777777777737</v>
       </c>
       <c r="B305" s="1">
-        <v>208.24175824175799</v>
+        <v>229.67032967032901</v>
       </c>
       <c r="C305" s="1">
         <v>700</v>
@@ -3710,10 +3710,10 @@
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A306" s="1">
-        <v>5577.7777777777737</v>
+        <v>4880.3418803418763</v>
       </c>
       <c r="B306" s="1">
-        <v>229.67032967032901</v>
+        <v>236.26373626373601</v>
       </c>
       <c r="C306" s="1">
         <v>700</v>
@@ -3721,10 +3721,10 @@
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A307" s="1">
-        <v>4880.3418803418763</v>
+        <v>4210.2564102564047</v>
       </c>
       <c r="B307" s="1">
-        <v>236.26373626373601</v>
+        <v>241.75824175824101</v>
       </c>
       <c r="C307" s="1">
         <v>700</v>
@@ -3732,10 +3732,10 @@
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A308" s="1">
-        <v>4210.2564102564047</v>
+        <v>3471.7948717948716</v>
       </c>
       <c r="B308" s="1">
-        <v>241.75824175824101</v>
+        <v>247.25274725274701</v>
       </c>
       <c r="C308" s="1">
         <v>700</v>
@@ -3743,10 +3743,10 @@
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A309" s="1">
-        <v>3471.7948717948716</v>
+        <v>2528.2051282051289</v>
       </c>
       <c r="B309" s="1">
-        <v>247.25274725274701</v>
+        <v>248.35164835164801</v>
       </c>
       <c r="C309" s="1">
         <v>700</v>
@@ -3754,10 +3754,10 @@
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A310" s="1">
-        <v>2528.2051282051289</v>
+        <v>1680.3418803418733</v>
       </c>
       <c r="B310" s="1">
-        <v>248.35164835164801</v>
+        <v>240.65934065933999</v>
       </c>
       <c r="C310" s="1">
         <v>700</v>
@@ -3765,10 +3765,10 @@
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A311" s="1">
-        <v>1680.3418803418733</v>
+        <v>217.09401709401772</v>
       </c>
       <c r="B311" s="1">
-        <v>240.65934065933999</v>
+        <v>226.923076923076</v>
       </c>
       <c r="C311" s="1">
         <v>700</v>
@@ -3776,10 +3776,10 @@
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A312" s="1">
-        <v>217.09401709401772</v>
+        <v>-931.62393162392732</v>
       </c>
       <c r="B312" s="1">
-        <v>226.923076923076</v>
+        <v>210.98901098901001</v>
       </c>
       <c r="C312" s="1">
         <v>700</v>
@@ -3787,10 +3787,10 @@
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A313" s="1">
-        <v>-931.62393162392732</v>
+        <v>-1533.3333333333294</v>
       </c>
       <c r="B313" s="1">
-        <v>210.98901098901001</v>
+        <v>195.60439560439499</v>
       </c>
       <c r="C313" s="1">
         <v>700</v>
@@ -3798,10 +3798,10 @@
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A314" s="1">
-        <v>-1533.3333333333294</v>
+        <v>-2353.8461538461502</v>
       </c>
       <c r="B314" s="1">
-        <v>195.60439560439499</v>
+        <v>170.32967032966999</v>
       </c>
       <c r="C314" s="1">
         <v>700</v>
@@ -3809,10 +3809,10 @@
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A315" s="1">
-        <v>-2353.8461538461502</v>
+        <v>-2695.7264957264902</v>
       </c>
       <c r="B315" s="1">
-        <v>170.32967032966999</v>
+        <v>138.461538461538</v>
       </c>
       <c r="C315" s="1">
         <v>700</v>
@@ -3820,10 +3820,10 @@
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A316" s="1">
-        <v>-2695.7264957264902</v>
+        <v>-2791.4529914529862</v>
       </c>
       <c r="B316" s="1">
-        <v>138.461538461538</v>
+        <v>104.395604395604</v>
       </c>
       <c r="C316" s="1">
         <v>700</v>
@@ -3831,10 +3831,10 @@
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A317" s="1">
-        <v>-2791.4529914529862</v>
+        <v>-2572.6495726495677</v>
       </c>
       <c r="B317" s="1">
-        <v>104.395604395604</v>
+        <v>73.626373626373606</v>
       </c>
       <c r="C317" s="1">
         <v>700</v>
@@ -3842,10 +3842,10 @@
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A318" s="1">
-        <v>-2572.6495726495677</v>
+        <v>-2107.6923076923053</v>
       </c>
       <c r="B318" s="1">
-        <v>73.626373626373606</v>
+        <v>45.604395604395499</v>
       </c>
       <c r="C318" s="1">
         <v>700</v>
@@ -3853,10 +3853,10 @@
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A319" s="1">
-        <v>-2107.6923076923053</v>
+        <v>-1615.384615384608</v>
       </c>
       <c r="B319" s="1">
-        <v>45.604395604395499</v>
+        <v>30.769230769230699</v>
       </c>
       <c r="C319" s="1">
         <v>700</v>
@@ -3864,10 +3864,10 @@
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A320" s="1">
-        <v>-1615.384615384608</v>
+        <v>-917.9487179487096</v>
       </c>
       <c r="B320" s="1">
-        <v>30.769230769230699</v>
+        <v>14.8351648351648</v>
       </c>
       <c r="C320" s="1">
         <v>700</v>
@@ -3875,10 +3875,10 @@
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A321" s="1">
-        <v>-917.9487179487096</v>
+        <v>-111.1111111111104</v>
       </c>
       <c r="B321" s="1">
-        <v>14.8351648351648</v>
+        <v>9.8901098901098905</v>
       </c>
       <c r="C321" s="1">
         <v>700</v>
@@ -3886,18 +3886,18 @@
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A322" s="1">
-        <v>-111.1111111111104</v>
+        <v>586.32478632478694</v>
       </c>
       <c r="B322" s="1">
-        <v>9.8901098901098905</v>
+        <v>0</v>
       </c>
       <c r="C322" s="1">
-        <v>700</v>
+        <v>800</v>
       </c>
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A323" s="1">
-        <v>586.32478632478694</v>
+        <v>1762.3931623931608</v>
       </c>
       <c r="B323" s="1">
         <v>0</v>
@@ -3908,7 +3908,7 @@
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A324" s="1">
-        <v>1762.3931623931608</v>
+        <v>3294.0170940170879</v>
       </c>
       <c r="B324" s="1">
         <v>0</v>
@@ -3919,7 +3919,7 @@
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A325" s="1">
-        <v>3294.0170940170879</v>
+        <v>4675.2136752136666</v>
       </c>
       <c r="B325" s="1">
         <v>0</v>
@@ -3930,7 +3930,7 @@
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A326" s="1">
-        <v>4675.2136752136666</v>
+        <v>5441.0256410256343</v>
       </c>
       <c r="B326" s="1">
         <v>0</v>
@@ -3941,10 +3941,10 @@
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A327" s="1">
-        <v>5441.0256410256343</v>
+        <v>6070.0854700854634</v>
       </c>
       <c r="B327" s="1">
-        <v>0</v>
+        <v>3.2967032967032899</v>
       </c>
       <c r="C327" s="1">
         <v>800</v>
@@ -3952,10 +3952,10 @@
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A328" s="1">
-        <v>6070.0854700854634</v>
+        <v>6726.4957264957266</v>
       </c>
       <c r="B328" s="1">
-        <v>3.2967032967032899</v>
+        <v>6.0439560439560296</v>
       </c>
       <c r="C328" s="1">
         <v>800</v>
@@ -3963,10 +3963,10 @@
     </row>
     <row r="329" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A329" s="1">
-        <v>6726.4957264957266</v>
+        <v>7205.1282051282069</v>
       </c>
       <c r="B329" s="1">
-        <v>6.0439560439560296</v>
+        <v>15.934065934065901</v>
       </c>
       <c r="C329" s="1">
         <v>800</v>
@@ -3974,10 +3974,10 @@
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A330" s="1">
-        <v>7205.1282051282069</v>
+        <v>7765.8119658119649</v>
       </c>
       <c r="B330" s="1">
-        <v>15.934065934065901</v>
+        <v>39.010989010988901</v>
       </c>
       <c r="C330" s="1">
         <v>800</v>
@@ -3985,10 +3985,10 @@
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A331" s="1">
-        <v>7765.8119658119649</v>
+        <v>8203.4188034188028</v>
       </c>
       <c r="B331" s="1">
-        <v>39.010989010988901</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C331" s="1">
         <v>800</v>
@@ -3996,10 +3996,10 @@
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A332" s="1">
-        <v>8203.4188034188028</v>
+        <v>8176.0683760683751</v>
       </c>
       <c r="B332" s="1">
-        <v>70.329670329670293</v>
+        <v>160.43956043956001</v>
       </c>
       <c r="C332" s="1">
         <v>800</v>
@@ -4007,10 +4007,10 @@
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A333" s="1">
-        <v>8176.0683760683751</v>
+        <v>7341.8803418803382</v>
       </c>
       <c r="B333" s="1">
-        <v>160.43956043956001</v>
+        <v>205.49450549450501</v>
       </c>
       <c r="C333" s="1">
         <v>800</v>
@@ -4018,10 +4018,10 @@
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A334" s="1">
-        <v>7341.8803418803382</v>
+        <v>6070.0854700854634</v>
       </c>
       <c r="B334" s="1">
-        <v>205.49450549450501</v>
+        <v>236.26373626373601</v>
       </c>
       <c r="C334" s="1">
         <v>800</v>
@@ -4029,10 +4029,10 @@
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A335" s="1">
-        <v>6070.0854700854634</v>
+        <v>4866.666666666667</v>
       </c>
       <c r="B335" s="1">
-        <v>236.26373626373601</v>
+        <v>249.450549450549</v>
       </c>
       <c r="C335" s="1">
         <v>800</v>
@@ -4040,10 +4040,10 @@
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A336" s="1">
-        <v>4866.666666666667</v>
+        <v>4264.9572649572656</v>
       </c>
       <c r="B336" s="1">
-        <v>249.450549450549</v>
+        <v>253.29670329670299</v>
       </c>
       <c r="C336" s="1">
         <v>800</v>
@@ -4051,7 +4051,7 @@
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A337" s="1">
-        <v>4264.9572649572656</v>
+        <v>1694.0170940170908</v>
       </c>
       <c r="B337" s="1">
         <v>253.29670329670299</v>
@@ -4062,10 +4062,10 @@
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A338" s="1">
-        <v>1694.0170940170908</v>
+        <v>1037.6068376068372</v>
       </c>
       <c r="B338" s="1">
-        <v>253.29670329670299</v>
+        <v>247.80219780219701</v>
       </c>
       <c r="C338" s="1">
         <v>800</v>
@@ -4073,10 +4073,10 @@
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A339" s="1">
-        <v>1037.6068376068372</v>
+        <v>162.39316239316275</v>
       </c>
       <c r="B339" s="1">
-        <v>247.80219780219701</v>
+        <v>237.362637362637</v>
       </c>
       <c r="C339" s="1">
         <v>800</v>
@@ -4084,10 +4084,10 @@
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A340" s="1">
-        <v>162.39316239316275</v>
+        <v>-576.06837606836962</v>
       </c>
       <c r="B340" s="1">
-        <v>237.362637362637</v>
+        <v>231.868131868131</v>
       </c>
       <c r="C340" s="1">
         <v>800</v>
@@ -4095,10 +4095,10 @@
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A341" s="1">
-        <v>-576.06837606836962</v>
+        <v>-1054.7008547008493</v>
       </c>
       <c r="B341" s="1">
-        <v>231.868131868131</v>
+        <v>224.175824175824</v>
       </c>
       <c r="C341" s="1">
         <v>800</v>
@@ -4106,10 +4106,10 @@
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A342" s="1">
-        <v>-1054.7008547008493</v>
+        <v>-1629.0598290598255</v>
       </c>
       <c r="B342" s="1">
-        <v>224.175824175824</v>
+        <v>210.98901098901001</v>
       </c>
       <c r="C342" s="1">
         <v>800</v>
@@ -4117,10 +4117,10 @@
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A343" s="1">
-        <v>-1629.0598290598255</v>
+        <v>-2135.0427350427317</v>
       </c>
       <c r="B343" s="1">
-        <v>210.98901098901001</v>
+        <v>194.505494505494</v>
       </c>
       <c r="C343" s="1">
         <v>800</v>
@@ -4128,10 +4128,10 @@
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A344" s="1">
-        <v>-2135.0427350427317</v>
+        <v>-2723.0769230769165</v>
       </c>
       <c r="B344" s="1">
-        <v>194.505494505494</v>
+        <v>171.42857142857099</v>
       </c>
       <c r="C344" s="1">
         <v>800</v>
@@ -4139,10 +4139,10 @@
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A345" s="1">
-        <v>-2723.0769230769165</v>
+        <v>-2969.2307692307695</v>
       </c>
       <c r="B345" s="1">
-        <v>171.42857142857099</v>
+        <v>148.35164835164801</v>
       </c>
       <c r="C345" s="1">
         <v>800</v>
@@ -4153,7 +4153,7 @@
         <v>-2969.2307692307695</v>
       </c>
       <c r="B346" s="1">
-        <v>148.35164835164801</v>
+        <v>84.065934065934002</v>
       </c>
       <c r="C346" s="1">
         <v>800</v>
@@ -4161,10 +4161,10 @@
     </row>
     <row r="347" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A347" s="1">
-        <v>-2969.2307692307695</v>
+        <v>-2791.4529914529862</v>
       </c>
       <c r="B347" s="1">
-        <v>84.065934065934002</v>
+        <v>59.890109890109898</v>
       </c>
       <c r="C347" s="1">
         <v>800</v>
@@ -4172,10 +4172,10 @@
     </row>
     <row r="348" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A348" s="1">
-        <v>-2791.4529914529862</v>
+        <v>-2435.8974358974283</v>
       </c>
       <c r="B348" s="1">
-        <v>59.890109890109898</v>
+        <v>40.109890109890102</v>
       </c>
       <c r="C348" s="1">
         <v>800</v>
@@ -4183,10 +4183,10 @@
     </row>
     <row r="349" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A349" s="1">
-        <v>-2435.8974358974283</v>
+        <v>-1943.5897435897396</v>
       </c>
       <c r="B349" s="1">
-        <v>40.109890109890102</v>
+        <v>23.076923076922998</v>
       </c>
       <c r="C349" s="1">
         <v>800</v>
@@ -4194,10 +4194,10 @@
     </row>
     <row r="350" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A350" s="1">
-        <v>-1943.5897435897396</v>
+        <v>-1396.5811965811897</v>
       </c>
       <c r="B350" s="1">
-        <v>23.076923076922998</v>
+        <v>10.439560439560401</v>
       </c>
       <c r="C350" s="1">
         <v>800</v>
@@ -4205,23 +4205,12 @@
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A351" s="1">
-        <v>-1396.5811965811897</v>
+        <v>-658.11965811965661</v>
       </c>
       <c r="B351" s="1">
-        <v>10.439560439560401</v>
+        <v>1.6483516483516401</v>
       </c>
       <c r="C351" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="352" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A352" s="1">
-        <v>-658.11965811965661</v>
-      </c>
-      <c r="B352" s="1">
-        <v>1.6483516483516401</v>
-      </c>
-      <c r="C352" s="1">
         <v>800</v>
       </c>
     </row>

</xml_diff>

<commit_message>
BSFC map plot generator added
</commit_message>
<xml_diff>
--- a/НИРС2/hCVT model/BSFC.xlsx
+++ b/НИРС2/hCVT model/BSFC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Баунти\Diplom\НИРС2\hCVT model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4856BD-8C8E-4B16-8A40-67B75310EEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFF0996B-63EC-4849-8395-1444647984D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="2" r:id="rId1"/>
@@ -347,7 +347,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC654685-493D-4E65-B880-F8D174A5EE76}">
-  <dimension ref="A1:C351"/>
+  <dimension ref="A1:C286"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="8.7265625" style="1"/>
@@ -553,7 +553,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
-        <v>3512.8205128205063</v>
+        <v>3512.82051282051</v>
       </c>
       <c r="B19" s="1">
         <v>109.890109890109</v>
@@ -564,7 +564,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
-        <v>3211.9658119658093</v>
+        <v>3211.9658119658102</v>
       </c>
       <c r="B20" s="1">
         <v>115.934065934065</v>
@@ -575,7 +575,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
-        <v>2801.7094017093991</v>
+        <v>2801.7094017094</v>
       </c>
       <c r="B21" s="1">
         <v>119.780219780219</v>
@@ -586,7 +586,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
-        <v>2555.5555555555547</v>
+        <v>2555.5555555555502</v>
       </c>
       <c r="B22" s="1">
         <v>124.72527472527401</v>
@@ -597,7 +597,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
-        <v>2104.2735042735012</v>
+        <v>2104.2735042734998</v>
       </c>
       <c r="B23" s="1">
         <v>119.780219780219</v>
@@ -608,7 +608,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
-        <v>1707.6923076922997</v>
+        <v>1707.6923076922999</v>
       </c>
       <c r="B24" s="1">
         <v>118.681318681318</v>
@@ -619,7 +619,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
-        <v>1242.7350427350432</v>
+        <v>1242.73504273504</v>
       </c>
       <c r="B25" s="1">
         <v>109.890109890109</v>
@@ -630,7 +630,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
-        <v>846.15384615384608</v>
+        <v>846.15384615384596</v>
       </c>
       <c r="B26" s="1">
         <v>98.351648351648294</v>
@@ -652,7 +652,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
-        <v>463.24786324786385</v>
+        <v>463.24786324786299</v>
       </c>
       <c r="B28" s="1">
         <v>87.912087912087898</v>
@@ -663,7 +663,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
-        <v>818.80341880341905</v>
+        <v>818.80341880341803</v>
       </c>
       <c r="B29" s="1">
         <v>80.219780219780205</v>
@@ -674,10 +674,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
-        <v>1229.0598290598291</v>
+        <v>1475.2136752136701</v>
       </c>
       <c r="B30" s="1">
-        <v>78.021978021978001</v>
+        <v>76.373626373626294</v>
       </c>
       <c r="C30" s="1">
         <v>225</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
-        <v>1475.2136752136728</v>
+        <v>2186.3247863247798</v>
       </c>
       <c r="B31" s="1">
-        <v>76.373626373626294</v>
+        <v>80.219780219780205</v>
       </c>
       <c r="C31" s="1">
         <v>225</v>
@@ -696,10 +696,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
-        <v>2186.3247863247798</v>
+        <v>2993.1623931623899</v>
       </c>
       <c r="B32" s="1">
-        <v>80.219780219780205</v>
+        <v>87.912087912087898</v>
       </c>
       <c r="C32" s="1">
         <v>225</v>
@@ -707,21 +707,21 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
-        <v>2993.1623931623917</v>
+        <v>4100.8547008547002</v>
       </c>
       <c r="B33" s="1">
-        <v>87.912087912087898</v>
+        <v>100</v>
       </c>
       <c r="C33" s="1">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
-        <v>4100.8547008547002</v>
+        <v>3977.7777777777701</v>
       </c>
       <c r="B34" s="1">
-        <v>100</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C34" s="1">
         <v>230</v>
@@ -729,10 +729,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
-        <v>3977.7777777777774</v>
+        <v>3950.4273504273501</v>
       </c>
       <c r="B35" s="1">
-        <v>109.890109890109</v>
+        <v>119.780219780219</v>
       </c>
       <c r="C35" s="1">
         <v>230</v>
@@ -740,10 +740,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
-        <v>3950.4273504273428</v>
+        <v>3540.17094017094</v>
       </c>
       <c r="B36" s="1">
-        <v>119.780219780219</v>
+        <v>129.12087912087901</v>
       </c>
       <c r="C36" s="1">
         <v>230</v>
@@ -751,10 +751,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
-        <v>3540.1709401709322</v>
+        <v>3006.8376068376001</v>
       </c>
       <c r="B37" s="1">
-        <v>129.12087912087901</v>
+        <v>134.06593406593399</v>
       </c>
       <c r="C37" s="1">
         <v>230</v>
@@ -762,10 +762,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
-        <v>3006.8376068376001</v>
+        <v>1694.0170940170899</v>
       </c>
       <c r="B38" s="1">
-        <v>134.06593406593399</v>
+        <v>129.67032967032901</v>
       </c>
       <c r="C38" s="1">
         <v>230</v>
@@ -773,10 +773,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
-        <v>2788.0341880341816</v>
+        <v>818.80341880341803</v>
       </c>
       <c r="B39" s="1">
-        <v>139.56043956043899</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C39" s="1">
         <v>230</v>
@@ -784,10 +784,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
-        <v>2569.2307692307636</v>
+        <v>326.49572649572599</v>
       </c>
       <c r="B40" s="1">
-        <v>139.56043956043899</v>
+        <v>105.49450549450501</v>
       </c>
       <c r="C40" s="1">
         <v>230</v>
@@ -795,10 +795,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
-        <v>1694.0170940170908</v>
+        <v>148.71794871794799</v>
       </c>
       <c r="B41" s="1">
-        <v>129.67032967032901</v>
+        <v>91.758241758241695</v>
       </c>
       <c r="C41" s="1">
         <v>230</v>
@@ -806,10 +806,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
-        <v>818.80341880341905</v>
+        <v>312.82051282051202</v>
       </c>
       <c r="B42" s="1">
-        <v>109.890109890109</v>
+        <v>79.120879120879096</v>
       </c>
       <c r="C42" s="1">
         <v>230</v>
@@ -817,10 +817,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
-        <v>326.49572649572684</v>
+        <v>805.12820512820497</v>
       </c>
       <c r="B43" s="1">
-        <v>105.49450549450501</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C43" s="1">
         <v>230</v>
@@ -828,10 +828,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
-        <v>148.71794871794884</v>
+        <v>1762.3931623931601</v>
       </c>
       <c r="B44" s="1">
-        <v>91.758241758241695</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C44" s="1">
         <v>230</v>
@@ -839,7 +839,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
-        <v>312.82051282051287</v>
+        <v>3034.1880341880301</v>
       </c>
       <c r="B45" s="1">
         <v>79.120879120879096</v>
@@ -850,10 +850,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
-        <v>805.12820512820508</v>
+        <v>3608.5470085470001</v>
       </c>
       <c r="B46" s="1">
-        <v>70.329670329670293</v>
+        <v>87.912087912087898</v>
       </c>
       <c r="C46" s="1">
         <v>230</v>
@@ -861,10 +861,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
-        <v>1037.6068376068372</v>
+        <v>3868.3760683760602</v>
       </c>
       <c r="B47" s="1">
-        <v>69.780219780219696</v>
+        <v>89.560439560439505</v>
       </c>
       <c r="C47" s="1">
         <v>230</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
-        <v>1762.3931623931608</v>
+        <v>2131.6239316239298</v>
       </c>
       <c r="B48" s="1">
-        <v>70.329670329670293</v>
+        <v>134.06593406593399</v>
       </c>
       <c r="C48" s="1">
         <v>230</v>
@@ -883,10 +883,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
-        <v>3034.188034188026</v>
+        <v>1256.41025641025</v>
       </c>
       <c r="B49" s="1">
-        <v>79.120879120879096</v>
+        <v>119.780219780219</v>
       </c>
       <c r="C49" s="1">
         <v>230</v>
@@ -894,10 +894,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
-        <v>3608.547008547002</v>
+        <v>2541.88034188034</v>
       </c>
       <c r="B50" s="1">
-        <v>87.912087912087898</v>
+        <v>139.56043956043899</v>
       </c>
       <c r="C50" s="1">
         <v>230</v>
@@ -905,10 +905,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
-        <v>3868.3760683760638</v>
+        <v>2801.7094017094</v>
       </c>
       <c r="B51" s="1">
-        <v>89.560439560439505</v>
+        <v>139.56043956043899</v>
       </c>
       <c r="C51" s="1">
         <v>230</v>
@@ -916,32 +916,32 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
-        <v>2131.6239316239271</v>
+        <v>2788.0341880341798</v>
       </c>
       <c r="B52" s="1">
-        <v>134.06593406593399</v>
+        <v>70.879120879120805</v>
       </c>
       <c r="C52" s="1">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
-        <v>1256.4102564102564</v>
+        <v>3635.8974358974301</v>
       </c>
       <c r="B53" s="1">
-        <v>119.780219780219</v>
+        <v>79.670329670329593</v>
       </c>
       <c r="C53" s="1">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
-        <v>2788.0341880341816</v>
+        <v>4114.5299145299095</v>
       </c>
       <c r="B54" s="1">
-        <v>70.879120879120805</v>
+        <v>86.813186813186803</v>
       </c>
       <c r="C54" s="1">
         <v>235</v>
@@ -949,10 +949,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
-        <v>3635.8974358974283</v>
+        <v>4538.4615384615299</v>
       </c>
       <c r="B55" s="1">
-        <v>79.670329670329593</v>
+        <v>99.450549450549403</v>
       </c>
       <c r="C55" s="1">
         <v>235</v>
@@ -960,10 +960,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
-        <v>4114.5299145299086</v>
+        <v>4401.7094017093996</v>
       </c>
       <c r="B56" s="1">
-        <v>86.813186813186803</v>
+        <v>114.28571428571399</v>
       </c>
       <c r="C56" s="1">
         <v>235</v>
@@ -971,10 +971,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
-        <v>4538.4615384615354</v>
+        <v>4087.17948717948</v>
       </c>
       <c r="B57" s="1">
-        <v>99.450549450549403</v>
+        <v>129.67032967032901</v>
       </c>
       <c r="C57" s="1">
         <v>235</v>
@@ -982,10 +982,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
-        <v>4401.7094017093959</v>
+        <v>3225.64102564102</v>
       </c>
       <c r="B58" s="1">
-        <v>114.28571428571399</v>
+        <v>141.75824175824101</v>
       </c>
       <c r="C58" s="1">
         <v>235</v>
@@ -993,10 +993,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
-        <v>4087.1794871794823</v>
+        <v>2829.05982905982</v>
       </c>
       <c r="B59" s="1">
-        <v>129.67032967032901</v>
+        <v>153.84615384615299</v>
       </c>
       <c r="C59" s="1">
         <v>235</v>
@@ -1004,10 +1004,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
-        <v>3225.6410256410181</v>
+        <v>2405.1282051282001</v>
       </c>
       <c r="B60" s="1">
-        <v>141.75824175824101</v>
+        <v>153.84615384615299</v>
       </c>
       <c r="C60" s="1">
         <v>235</v>
@@ -1015,10 +1015,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
-        <v>2829.0598290598255</v>
+        <v>2104.2735042734998</v>
       </c>
       <c r="B61" s="1">
-        <v>153.84615384615299</v>
+        <v>141.20879120879101</v>
       </c>
       <c r="C61" s="1">
         <v>235</v>
@@ -1026,10 +1026,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
-        <v>2405.1282051281978</v>
+        <v>545.29914529914504</v>
       </c>
       <c r="B62" s="1">
-        <v>153.84615384615299</v>
+        <v>115.384615384615</v>
       </c>
       <c r="C62" s="1">
         <v>235</v>
@@ -1037,10 +1037,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
-        <v>2104.2735042735012</v>
+        <v>-165.811965811965</v>
       </c>
       <c r="B63" s="1">
-        <v>141.20879120879101</v>
+        <v>100</v>
       </c>
       <c r="C63" s="1">
         <v>235</v>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
-        <v>1666.6666666666647</v>
+        <v>-1.70940170940139</v>
       </c>
       <c r="B64" s="1">
-        <v>135.16483516483501</v>
+        <v>79.670329670329593</v>
       </c>
       <c r="C64" s="1">
         <v>235</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
-        <v>1461.5384615384614</v>
+        <v>818.80341880341803</v>
       </c>
       <c r="B65" s="1">
-        <v>129.67032967032901</v>
+        <v>65.384615384615302</v>
       </c>
       <c r="C65" s="1">
         <v>235</v>
@@ -1070,10 +1070,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
-        <v>1037.6068376068372</v>
+        <v>1830.76923076923</v>
       </c>
       <c r="B66" s="1">
-        <v>123.626373626373</v>
+        <v>65.934065934065899</v>
       </c>
       <c r="C66" s="1">
         <v>235</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
-        <v>818.80341880341905</v>
+        <v>3800</v>
       </c>
       <c r="B67" s="1">
-        <v>117.58241758241699</v>
+        <v>136.81318681318601</v>
       </c>
       <c r="C67" s="1">
         <v>235</v>
@@ -1092,10 +1092,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
-        <v>545.29914529914561</v>
+        <v>1133.3333333333301</v>
       </c>
       <c r="B68" s="1">
-        <v>115.384615384615</v>
+        <v>124.72527472527401</v>
       </c>
       <c r="C68" s="1">
         <v>235</v>
@@ -1103,10 +1103,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
-        <v>94.017094017094678</v>
+        <v>1625.64102564102</v>
       </c>
       <c r="B69" s="1">
-        <v>109.890109890109</v>
+        <v>134.61538461538399</v>
       </c>
       <c r="C69" s="1">
         <v>235</v>
@@ -1114,98 +1114,98 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
-        <v>-165.81196581196536</v>
+        <v>3635.8974358974301</v>
       </c>
       <c r="B70" s="1">
-        <v>100</v>
+        <v>74.725274725274701</v>
       </c>
       <c r="C70" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
-        <v>-1.709401709401277</v>
+        <v>4210.2564102564102</v>
       </c>
       <c r="B71" s="1">
         <v>79.670329670329593</v>
       </c>
       <c r="C71" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
-        <v>340.17094017094081</v>
+        <v>4743.5897435897396</v>
       </c>
       <c r="B72" s="1">
-        <v>72.527472527472497</v>
+        <v>105.49450549450501</v>
       </c>
       <c r="C72" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
-        <v>818.80341880341905</v>
+        <v>4620.5128205128203</v>
       </c>
       <c r="B73" s="1">
-        <v>65.384615384615302</v>
+        <v>130.21978021978001</v>
       </c>
       <c r="C73" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
-        <v>1133.3333333333333</v>
+        <v>3882.0512820512799</v>
       </c>
       <c r="B74" s="1">
-        <v>65.934065934065899</v>
+        <v>143.956043956043</v>
       </c>
       <c r="C74" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
-        <v>1830.7692307692305</v>
+        <v>3335.0427350427299</v>
       </c>
       <c r="B75" s="1">
-        <v>65.934065934065899</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C75" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
-        <v>2254.700854700849</v>
+        <v>3088.88888888888</v>
       </c>
       <c r="B76" s="1">
-        <v>67.582417582417506</v>
+        <v>159.34065934065899</v>
       </c>
       <c r="C76" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
-        <v>3799.9999999999941</v>
+        <v>2405.1282051282001</v>
       </c>
       <c r="B77" s="1">
-        <v>136.81318681318601</v>
+        <v>162.087912087912</v>
       </c>
       <c r="C77" s="1">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
-        <v>3047.8632478632435</v>
+        <v>2035.8974358974299</v>
       </c>
       <c r="B78" s="1">
-        <v>67.582417582417506</v>
+        <v>153.29670329670299</v>
       </c>
       <c r="C78" s="1">
         <v>240</v>
@@ -1213,10 +1213,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
-        <v>3635.8974358974283</v>
+        <v>1639.3162393162299</v>
       </c>
       <c r="B79" s="1">
-        <v>74.725274725274701</v>
+        <v>144.505494505494</v>
       </c>
       <c r="C79" s="1">
         <v>240</v>
@@ -1224,10 +1224,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
-        <v>4210.2564102564047</v>
+        <v>1119.6581196581201</v>
       </c>
       <c r="B80" s="1">
-        <v>79.670329670329593</v>
+        <v>130.76923076923001</v>
       </c>
       <c r="C80" s="1">
         <v>240</v>
@@ -1235,10 +1235,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
-        <v>4483.7606837606836</v>
+        <v>613.67521367521294</v>
       </c>
       <c r="B81" s="1">
-        <v>89.560439560439505</v>
+        <v>123.626373626373</v>
       </c>
       <c r="C81" s="1">
         <v>240</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
-        <v>4743.5897435897368</v>
+        <v>-1.70940170940139</v>
       </c>
       <c r="B82" s="1">
-        <v>105.49450549450501</v>
+        <v>118.681318681318</v>
       </c>
       <c r="C82" s="1">
         <v>240</v>
@@ -1257,10 +1257,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
-        <v>4729.9145299145284</v>
+        <v>-411.96581196581201</v>
       </c>
       <c r="B83" s="1">
-        <v>121.428571428571</v>
+        <v>98.901098901098905</v>
       </c>
       <c r="C83" s="1">
         <v>240</v>
@@ -1268,10 +1268,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
-        <v>4620.5128205128149</v>
+        <v>-97.435897435897402</v>
       </c>
       <c r="B84" s="1">
-        <v>130.21978021978001</v>
+        <v>74.725274725274701</v>
       </c>
       <c r="C84" s="1">
         <v>240</v>
@@ -1279,10 +1279,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
-        <v>4210.2564102564047</v>
+        <v>367.52136752136698</v>
       </c>
       <c r="B85" s="1">
-        <v>140.10989010988999</v>
+        <v>64.835164835164804</v>
       </c>
       <c r="C85" s="1">
         <v>240</v>
@@ -1290,10 +1290,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
-        <v>3882.0512820512813</v>
+        <v>1037.6068376068299</v>
       </c>
       <c r="B86" s="1">
-        <v>143.956043956043</v>
+        <v>62.087912087912002</v>
       </c>
       <c r="C86" s="1">
         <v>240</v>
@@ -1301,10 +1301,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
-        <v>3335.0427350427317</v>
+        <v>1871.79487179487</v>
       </c>
       <c r="B87" s="1">
-        <v>149.450549450549</v>
+        <v>61.538461538461497</v>
       </c>
       <c r="C87" s="1">
         <v>240</v>
@@ -1312,10 +1312,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
-        <v>3088.8888888888869</v>
+        <v>2623.9316239316199</v>
       </c>
       <c r="B88" s="1">
-        <v>159.34065934065899</v>
+        <v>64.285714285714207</v>
       </c>
       <c r="C88" s="1">
         <v>240</v>
@@ -1323,208 +1323,208 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
-        <v>2405.1282051281978</v>
+        <v>4524.7863247863197</v>
       </c>
       <c r="B89" s="1">
-        <v>162.087912087912</v>
+        <v>77.472527472527403</v>
       </c>
       <c r="C89" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
-        <v>2035.8974358974313</v>
+        <v>5085.4700854700804</v>
       </c>
       <c r="B90" s="1">
-        <v>153.29670329670299</v>
+        <v>90.109890109890102</v>
       </c>
       <c r="C90" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
-        <v>1912.8205128205091</v>
+        <v>5413.6752136752102</v>
       </c>
       <c r="B91" s="1">
-        <v>147.25274725274701</v>
+        <v>128.57142857142799</v>
       </c>
       <c r="C91" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
-        <v>1639.3162393162386</v>
+        <v>5495.7264957264897</v>
       </c>
       <c r="B92" s="1">
-        <v>144.505494505494</v>
+        <v>108.79120879120801</v>
       </c>
       <c r="C92" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
-        <v>1119.6581196581192</v>
+        <v>4948.7179487179401</v>
       </c>
       <c r="B93" s="1">
-        <v>130.76923076923001</v>
+        <v>140.65934065933999</v>
       </c>
       <c r="C93" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
-        <v>613.67521367521385</v>
+        <v>4333.3333333333303</v>
       </c>
       <c r="B94" s="1">
-        <v>123.626373626373</v>
+        <v>145.05494505494499</v>
       </c>
       <c r="C94" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
-        <v>-1.709401709401277</v>
+        <v>3581.1965811965802</v>
       </c>
       <c r="B95" s="1">
-        <v>118.681318681318</v>
+        <v>160.98901098901001</v>
       </c>
       <c r="C95" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
-        <v>-357.26495726495125</v>
+        <v>2596.5811965811899</v>
       </c>
       <c r="B96" s="1">
-        <v>107.692307692307</v>
+        <v>168.681318681318</v>
       </c>
       <c r="C96" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
-        <v>-411.96581196580371</v>
+        <v>1666.6666666666599</v>
       </c>
       <c r="B97" s="1">
-        <v>98.901098901098905</v>
+        <v>162.087912087912</v>
       </c>
       <c r="C97" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
-        <v>-370.94017094016863</v>
+        <v>996.58119658119597</v>
       </c>
       <c r="B98" s="1">
-        <v>87.912087912087898</v>
+        <v>146.15384615384599</v>
       </c>
       <c r="C98" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
-        <v>-97.435897435897346</v>
+        <v>162.39316239316199</v>
       </c>
       <c r="B99" s="1">
-        <v>74.725274725274701</v>
+        <v>128.57142857142799</v>
       </c>
       <c r="C99" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
-        <v>367.52136752136789</v>
+        <v>-452.99145299145198</v>
       </c>
       <c r="B100" s="1">
-        <v>64.835164835164804</v>
+        <v>117.58241758241699</v>
       </c>
       <c r="C100" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
-        <v>805.12820512820508</v>
+        <v>-630.76923076923094</v>
       </c>
       <c r="B101" s="1">
-        <v>62.087912087912002</v>
+        <v>98.901098901098905</v>
       </c>
       <c r="C101" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
-        <v>1037.6068376068372</v>
+        <v>-220.51282051282001</v>
       </c>
       <c r="B102" s="1">
-        <v>62.087912087912002</v>
+        <v>71.428571428571402</v>
       </c>
       <c r="C102" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
-        <v>1283.7606837606834</v>
+        <v>312.82051282051202</v>
       </c>
       <c r="B103" s="1">
-        <v>61.538461538461497</v>
+        <v>62.087912087912002</v>
       </c>
       <c r="C103" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
-        <v>1871.7948717948655</v>
+        <v>1037.6068376068299</v>
       </c>
       <c r="B104" s="1">
-        <v>61.538461538461497</v>
+        <v>58.241758241758198</v>
       </c>
       <c r="C104" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
-        <v>2295.7264957264933</v>
+        <v>2117.9487179487101</v>
       </c>
       <c r="B105" s="1">
-        <v>63.186813186813197</v>
+        <v>58.241758241758198</v>
       </c>
       <c r="C105" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
-        <v>2623.9316239316158</v>
+        <v>3198.29059829059</v>
       </c>
       <c r="B106" s="1">
-        <v>64.285714285714207</v>
+        <v>60.989010989011</v>
       </c>
       <c r="C106" s="1">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
-        <v>4524.7863247863188</v>
+        <v>3690.5982905982901</v>
       </c>
       <c r="B107" s="1">
-        <v>77.472527472527403</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C107" s="1">
         <v>245</v>
@@ -1532,2685 +1532,1970 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
-        <v>4798.2905982905977</v>
+        <v>3280.3418803418799</v>
       </c>
       <c r="B108" s="1">
-        <v>86.263736263736206</v>
+        <v>57.142857142857103</v>
       </c>
       <c r="C108" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
-        <v>5085.4700854700859</v>
+        <v>4100.8547008547002</v>
       </c>
       <c r="B109" s="1">
-        <v>90.109890109890102</v>
+        <v>59.890109890109898</v>
       </c>
       <c r="C109" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
-        <v>5181.1965811965729</v>
+        <v>5878.6324786324703</v>
       </c>
       <c r="B110" s="1">
-        <v>100</v>
+        <v>91.208791208791197</v>
       </c>
       <c r="C110" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
-        <v>5413.6752136752084</v>
+        <v>6138.4615384615299</v>
       </c>
       <c r="B111" s="1">
-        <v>128.57142857142799</v>
+        <v>123.626373626373</v>
       </c>
       <c r="C111" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
-        <v>5495.7264957264952</v>
+        <v>5386.3247863247798</v>
       </c>
       <c r="B112" s="1">
-        <v>108.79120879120801</v>
+        <v>143.406593406593</v>
       </c>
       <c r="C112" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
-        <v>5290.5982905982864</v>
+        <v>4675.2136752136703</v>
       </c>
       <c r="B113" s="1">
-        <v>135.71428571428501</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C113" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
-        <v>4333.3333333333267</v>
+        <v>3882.0512820512799</v>
       </c>
       <c r="B114" s="1">
-        <v>145.05494505494499</v>
+        <v>167.58241758241701</v>
       </c>
       <c r="C114" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
-        <v>3717.9487179487155</v>
+        <v>2952.1367521367501</v>
       </c>
       <c r="B115" s="1">
-        <v>153.29670329670299</v>
+        <v>178.57142857142799</v>
       </c>
       <c r="C115" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
-        <v>3581.1965811965761</v>
+        <v>1830.76923076923</v>
       </c>
       <c r="B116" s="1">
-        <v>160.98901098901001</v>
+        <v>174.175824175824</v>
       </c>
       <c r="C116" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
-        <v>3088.8888888888869</v>
+        <v>1064.9572649572599</v>
       </c>
       <c r="B117" s="1">
-        <v>168.131868131868</v>
+        <v>160.98901098901001</v>
       </c>
       <c r="C117" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
-        <v>2596.5811965811899</v>
+        <v>-535.04273504273397</v>
       </c>
       <c r="B118" s="1">
-        <v>168.681318681318</v>
+        <v>132.967032967032</v>
       </c>
       <c r="C118" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
-        <v>2076.9230769230753</v>
+        <v>-849.57264957264897</v>
       </c>
       <c r="B119" s="1">
-        <v>165.93406593406499</v>
+        <v>111.53846153846099</v>
       </c>
       <c r="C119" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
-        <v>1666.6666666666647</v>
+        <v>-740.17094017093996</v>
       </c>
       <c r="B120" s="1">
-        <v>162.087912087912</v>
+        <v>80.219780219780205</v>
       </c>
       <c r="C120" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
-        <v>1270.0854700854693</v>
+        <v>244.444444444444</v>
       </c>
       <c r="B121" s="1">
-        <v>151.648351648351</v>
+        <v>57.142857142857103</v>
       </c>
       <c r="C121" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
-        <v>996.5811965811962</v>
+        <v>1010.25641025641</v>
       </c>
       <c r="B122" s="1">
-        <v>146.15384615384599</v>
+        <v>53.846153846153797</v>
       </c>
       <c r="C122" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
-        <v>627.35042735042771</v>
+        <v>1830.76923076923</v>
       </c>
       <c r="B123" s="1">
-        <v>135.16483516483501</v>
+        <v>52.747252747252702</v>
       </c>
       <c r="C123" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
-        <v>162.39316239316275</v>
+        <v>326.49572649572599</v>
       </c>
       <c r="B124" s="1">
-        <v>128.57142857142799</v>
+        <v>147.80219780219701</v>
       </c>
       <c r="C124" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
-        <v>-452.9914529914472</v>
+        <v>4976.0683760683696</v>
       </c>
       <c r="B125" s="1">
-        <v>117.58241758241699</v>
+        <v>80.219780219780205</v>
       </c>
       <c r="C125" s="1">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
-        <v>-630.76923076923049</v>
+        <v>600</v>
       </c>
       <c r="B126" s="1">
-        <v>98.901098901098905</v>
+        <v>41.758241758241702</v>
       </c>
       <c r="C126" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
-        <v>-548.71794871794327</v>
+        <v>1735.0427350427301</v>
       </c>
       <c r="B127" s="1">
-        <v>82.967032967032907</v>
+        <v>42.857142857142797</v>
       </c>
       <c r="C127" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
-        <v>-220.51282051282033</v>
+        <v>2883.76068376068</v>
       </c>
       <c r="B128" s="1">
-        <v>71.428571428571402</v>
+        <v>44.505494505494497</v>
       </c>
       <c r="C128" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
-        <v>312.82051282051287</v>
+        <v>3964.1025641025599</v>
       </c>
       <c r="B129" s="1">
-        <v>62.087912087912002</v>
+        <v>47.252747252747199</v>
       </c>
       <c r="C129" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" s="1">
-        <v>777.77777777777806</v>
+        <v>4770.94017094017</v>
       </c>
       <c r="B130" s="1">
-        <v>58.241758241758198</v>
+        <v>49.450549450549403</v>
       </c>
       <c r="C130" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" s="1">
-        <v>1037.6068376068372</v>
+        <v>5413.6752136752102</v>
       </c>
       <c r="B131" s="1">
-        <v>58.241758241758198</v>
+        <v>53.296703296703299</v>
       </c>
       <c r="C131" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" s="1">
-        <v>1475.2136752136728</v>
+        <v>6370.94017094017</v>
       </c>
       <c r="B132" s="1">
-        <v>57.142857142857103</v>
+        <v>74.725274725274701</v>
       </c>
       <c r="C132" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" s="1">
-        <v>2117.9487179487187</v>
+        <v>6808.5470085469997</v>
       </c>
       <c r="B133" s="1">
-        <v>58.241758241758198</v>
+        <v>120.32967032966999</v>
       </c>
       <c r="C133" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" s="1">
-        <v>2829.0598290598255</v>
+        <v>3800</v>
       </c>
       <c r="B134" s="1">
-        <v>60.439560439560402</v>
+        <v>192.85714285714201</v>
       </c>
       <c r="C134" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" s="1">
-        <v>3198.2905982905918</v>
+        <v>1830.76923076923</v>
       </c>
       <c r="B135" s="1">
-        <v>60.989010989011</v>
+        <v>193.406593406593</v>
       </c>
       <c r="C135" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" s="1">
-        <v>3690.5982905982892</v>
+        <v>736.75213675213695</v>
       </c>
       <c r="B136" s="1">
-        <v>70.329670329670293</v>
+        <v>180.76923076923001</v>
       </c>
       <c r="C136" s="1">
-        <v>245</v>
+        <v>275</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" s="1">
-        <v>2705.9829059829035</v>
+        <v>-247.86324786324801</v>
       </c>
       <c r="B137" s="1">
-        <v>54.945054945054899</v>
+        <v>165.93406593406499</v>
       </c>
       <c r="C137" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" s="1">
-        <v>3280.3418803418795</v>
+        <v>-1136.7521367521299</v>
       </c>
       <c r="B138" s="1">
-        <v>57.142857142857103</v>
+        <v>146.15384615384599</v>
       </c>
       <c r="C138" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" s="1">
-        <v>4100.8547008547002</v>
+        <v>-1437.6068376068299</v>
       </c>
       <c r="B139" s="1">
-        <v>59.890109890109898</v>
+        <v>122.527472527472</v>
       </c>
       <c r="C139" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" s="1">
-        <v>4305.9829059829008</v>
+        <v>-1423.9316239316199</v>
       </c>
       <c r="B140" s="1">
-        <v>69.780219780219696</v>
+        <v>89.560439560439505</v>
       </c>
       <c r="C140" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" s="1">
-        <v>4565.8119658119622</v>
+        <v>-945.29914529914504</v>
       </c>
       <c r="B141" s="1">
-        <v>71.428571428571402</v>
+        <v>62.6373626373626</v>
       </c>
       <c r="C141" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" s="1">
-        <v>5099.1452991452943</v>
+        <v>80.341880341880298</v>
       </c>
       <c r="B142" s="1">
-        <v>81.868131868131798</v>
+        <v>43.406593406593402</v>
       </c>
       <c r="C142" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143" s="1">
-        <v>5878.6324786324712</v>
+        <v>4770.94017094017</v>
       </c>
       <c r="B143" s="1">
-        <v>91.208791208791197</v>
+        <v>181.868131868131</v>
       </c>
       <c r="C143" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" s="1">
-        <v>6152.1367521367501</v>
+        <v>6425.64102564102</v>
       </c>
       <c r="B144" s="1">
-        <v>104.395604395604</v>
+        <v>154.94505494505401</v>
       </c>
       <c r="C144" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145" s="1">
-        <v>6138.4615384615336</v>
+        <v>5632.4786324786301</v>
       </c>
       <c r="B145" s="1">
-        <v>123.626373626373</v>
+        <v>168.681318681318</v>
       </c>
       <c r="C145" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A146" s="1">
-        <v>5851.2820512820463</v>
+        <v>2870.0854700854702</v>
       </c>
       <c r="B146" s="1">
-        <v>136.26373626373601</v>
+        <v>200</v>
       </c>
       <c r="C146" s="1">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A147" s="1">
-        <v>5386.3247863247834</v>
+        <v>600</v>
       </c>
       <c r="B147" s="1">
-        <v>143.406593406593</v>
+        <v>38.461538461538403</v>
       </c>
       <c r="C147" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A148" s="1">
-        <v>4675.2136752136666</v>
+        <v>1967.5213675213599</v>
       </c>
       <c r="B148" s="1">
-        <v>149.450549450549</v>
+        <v>39.010989010988901</v>
       </c>
       <c r="C148" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A149" s="1">
-        <v>4182.9059829059788</v>
+        <v>3239.3162393162302</v>
       </c>
       <c r="B149" s="1">
-        <v>155.49450549450501</v>
+        <v>39.010989010988901</v>
       </c>
       <c r="C149" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A150" s="1">
-        <v>3882.0512820512813</v>
+        <v>5400</v>
       </c>
       <c r="B150" s="1">
-        <v>167.58241758241701</v>
+        <v>46.153846153846096</v>
       </c>
       <c r="C150" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A151" s="1">
-        <v>2952.1367521367479</v>
+        <v>5974.35897435897</v>
       </c>
       <c r="B151" s="1">
-        <v>178.57142857142799</v>
+        <v>60.439560439560402</v>
       </c>
       <c r="C151" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A152" s="1">
-        <v>1830.7692307692305</v>
+        <v>6835.8974358974301</v>
       </c>
       <c r="B152" s="1">
-        <v>174.175824175824</v>
+        <v>90.6593406593406</v>
       </c>
       <c r="C152" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A153" s="1">
-        <v>1064.9572649572642</v>
+        <v>7013.6752136752102</v>
       </c>
       <c r="B153" s="1">
-        <v>160.98901098901001</v>
+        <v>120.87912087911999</v>
       </c>
       <c r="C153" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A154" s="1">
-        <v>600</v>
+        <v>6781.1965811965802</v>
       </c>
       <c r="B154" s="1">
-        <v>151.098901098901</v>
+        <v>152.74725274725199</v>
       </c>
       <c r="C154" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A155" s="1">
-        <v>-535.04273504273465</v>
+        <v>6343.5897435897396</v>
       </c>
       <c r="B155" s="1">
-        <v>132.967032967032</v>
+        <v>167.03296703296701</v>
       </c>
       <c r="C155" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A156" s="1">
-        <v>-849.57264957264897</v>
+        <v>5755.5555555555502</v>
       </c>
       <c r="B156" s="1">
-        <v>111.53846153846099</v>
+        <v>174.72527472527401</v>
       </c>
       <c r="C156" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A157" s="1">
-        <v>-740.17094017093541</v>
+        <v>4770.94017094017</v>
       </c>
       <c r="B157" s="1">
-        <v>80.219780219780205</v>
+        <v>190.10989010988999</v>
       </c>
       <c r="C157" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158" s="1">
-        <v>-288.88888888888141</v>
+        <v>3964.1025641025599</v>
       </c>
       <c r="B158" s="1">
-        <v>66.483516483516397</v>
+        <v>200</v>
       </c>
       <c r="C158" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" s="1">
-        <v>244.4444444444448</v>
+        <v>3294.0170940170901</v>
       </c>
       <c r="B159" s="1">
-        <v>57.142857142857103</v>
+        <v>208.79120879120799</v>
       </c>
       <c r="C159" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160" s="1">
-        <v>600</v>
+        <v>2487.17948717948</v>
       </c>
       <c r="B160" s="1">
-        <v>54.945054945054899</v>
+        <v>208.24175824175799</v>
       </c>
       <c r="C160" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161" s="1">
-        <v>1010.2564102564102</v>
+        <v>1694.0170940170899</v>
       </c>
       <c r="B161" s="1">
-        <v>53.846153846153797</v>
+        <v>201.648351648351</v>
       </c>
       <c r="C161" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162" s="1">
-        <v>1830.7692307692305</v>
+        <v>449.57264957264903</v>
       </c>
       <c r="B162" s="1">
-        <v>52.747252747252702</v>
+        <v>186.81318681318601</v>
       </c>
       <c r="C162" s="1">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163" s="1">
-        <v>600</v>
+        <v>-439.31623931623898</v>
       </c>
       <c r="B163" s="1">
-        <v>41.758241758241702</v>
+        <v>171.97802197802099</v>
       </c>
       <c r="C163" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164" s="1">
-        <v>1735.0427350427346</v>
+        <v>-1314.52991452991</v>
       </c>
       <c r="B164" s="1">
-        <v>42.857142857142797</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C164" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" s="1">
-        <v>2883.7606837606777</v>
+        <v>-1588.03418803418</v>
       </c>
       <c r="B165" s="1">
-        <v>44.505494505494497</v>
+        <v>126.373626373626</v>
       </c>
       <c r="C165" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166" s="1">
-        <v>3964.1025641025599</v>
+        <v>-1588.03418803418</v>
       </c>
       <c r="B166" s="1">
-        <v>47.252747252747199</v>
+        <v>92.307692307692193</v>
       </c>
       <c r="C166" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167" s="1">
-        <v>4770.9401709401718</v>
+        <v>-1068.3760683760599</v>
       </c>
       <c r="B167" s="1">
-        <v>49.450549450549403</v>
+        <v>60.989010989011</v>
       </c>
       <c r="C167" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A168" s="1">
-        <v>5413.6752136752084</v>
+        <v>25.641025641025799</v>
       </c>
       <c r="B168" s="1">
-        <v>53.296703296703299</v>
+        <v>39.560439560439498</v>
       </c>
       <c r="C168" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169" s="1">
-        <v>5851.2820512820463</v>
+        <v>4360.6837606837598</v>
       </c>
       <c r="B169" s="1">
-        <v>63.186813186813197</v>
+        <v>43.406593406593402</v>
       </c>
       <c r="C169" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A170" s="1">
-        <v>6370.9401709401682</v>
+        <v>572.64957264957195</v>
       </c>
       <c r="B170" s="1">
-        <v>74.725274725274701</v>
+        <v>30.769230769230699</v>
       </c>
       <c r="C170" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A171" s="1">
-        <v>6685.4700854700832</v>
+        <v>5400</v>
       </c>
       <c r="B171" s="1">
-        <v>93.956043956043899</v>
+        <v>35.164835164835097</v>
       </c>
       <c r="C171" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A172" s="1">
-        <v>6808.5470085470051</v>
+        <v>7041.0256410256397</v>
       </c>
       <c r="B172" s="1">
-        <v>120.32967032966999</v>
+        <v>76.923076923076906</v>
       </c>
       <c r="C172" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A173" s="1">
-        <v>6589.7435897435862</v>
+        <v>4866.6666666666597</v>
       </c>
       <c r="B173" s="1">
-        <v>147.25274725274701</v>
+        <v>202.74725274725199</v>
       </c>
       <c r="C173" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A174" s="1">
-        <v>5823.9316239316186</v>
+        <v>3430.76923076923</v>
       </c>
       <c r="B174" s="1">
-        <v>164.83516483516399</v>
+        <v>219.780219780219</v>
       </c>
       <c r="C174" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A175" s="1">
-        <v>4948.7179487179455</v>
+        <v>2282.0512820512799</v>
       </c>
       <c r="B175" s="1">
-        <v>179.12087912087901</v>
+        <v>219.780219780219</v>
       </c>
       <c r="C175" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A176" s="1">
-        <v>3799.9999999999941</v>
+        <v>1174.35897435897</v>
       </c>
       <c r="B176" s="1">
-        <v>192.85714285714201</v>
+        <v>206.593406593406</v>
       </c>
       <c r="C176" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A177" s="1">
-        <v>3225.6410256410181</v>
+        <v>-179.48717948717899</v>
       </c>
       <c r="B177" s="1">
-        <v>200</v>
+        <v>189.01098901098899</v>
       </c>
       <c r="C177" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A178" s="1">
-        <v>2514.5299145299114</v>
+        <v>-1068.3760683760599</v>
       </c>
       <c r="B178" s="1">
-        <v>198.90109890109801</v>
+        <v>170.32967032966999</v>
       </c>
       <c r="C178" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A179" s="1">
-        <v>1830.7692307692305</v>
+        <v>-1683.76068376068</v>
       </c>
       <c r="B179" s="1">
-        <v>193.406593406593</v>
+        <v>149.450549450549</v>
       </c>
       <c r="C179" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A180" s="1">
-        <v>736.75213675213695</v>
+        <v>-1847.8632478632401</v>
       </c>
       <c r="B180" s="1">
-        <v>180.76923076923001</v>
+        <v>123.07692307692299</v>
       </c>
       <c r="C180" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A181" s="1">
-        <v>-247.86324786324747</v>
+        <v>-1888.88888888888</v>
       </c>
       <c r="B181" s="1">
-        <v>165.93406593406499</v>
+        <v>93.956043956043899</v>
       </c>
       <c r="C181" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A182" s="1">
-        <v>-1136.7521367521279</v>
+        <v>-1560.6837606837601</v>
       </c>
       <c r="B182" s="1">
-        <v>146.15384615384599</v>
+        <v>67.582417582417506</v>
       </c>
       <c r="C182" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A183" s="1">
-        <v>-1437.6068376068336</v>
+        <v>-863.24786324786305</v>
       </c>
       <c r="B183" s="1">
-        <v>122.527472527472</v>
+        <v>42.857142857142797</v>
       </c>
       <c r="C183" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A184" s="1">
-        <v>-1423.9316239316158</v>
+        <v>-1.70940170940139</v>
       </c>
       <c r="B184" s="1">
-        <v>89.560439560439505</v>
+        <v>31.3186813186813</v>
       </c>
       <c r="C184" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A185" s="1">
-        <v>-945.29914529914458</v>
+        <v>1584.61538461538</v>
       </c>
       <c r="B185" s="1">
-        <v>62.6373626373626</v>
+        <v>32.9670329670329</v>
       </c>
       <c r="C185" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A186" s="1">
-        <v>-425.64102564102109</v>
+        <v>2870.0854700854702</v>
       </c>
       <c r="B186" s="1">
-        <v>51.6483516483516</v>
+        <v>32.9670329670329</v>
       </c>
       <c r="C186" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A187" s="1">
-        <v>80.34188034188071</v>
+        <v>4223.9316239316204</v>
       </c>
       <c r="B187" s="1">
-        <v>43.406593406593402</v>
+        <v>32.9670329670329</v>
       </c>
       <c r="C187" s="1">
-        <v>275</v>
+        <v>400</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A188" s="1">
-        <v>600</v>
+        <v>5988.0341880341803</v>
       </c>
       <c r="B188" s="1">
-        <v>38.461538461538403</v>
+        <v>185.71428571428501</v>
       </c>
       <c r="C188" s="1">
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A189" s="1">
-        <v>1967.5213675213613</v>
+        <v>7027.3504273504204</v>
       </c>
       <c r="B189" s="1">
-        <v>39.010989010988901</v>
+        <v>160.98901098901001</v>
       </c>
       <c r="C189" s="1">
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A190" s="1">
-        <v>3239.3162393162356</v>
+        <v>7300.8547008547002</v>
       </c>
       <c r="B190" s="1">
-        <v>39.010989010988901</v>
+        <v>120.87912087911999</v>
       </c>
       <c r="C190" s="1">
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A191" s="1">
-        <v>4716.2393162393109</v>
+        <v>6288.8888888888796</v>
       </c>
       <c r="B191" s="1">
-        <v>43.956043956043899</v>
+        <v>52.197802197802098</v>
       </c>
       <c r="C191" s="1">
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A192" s="1">
-        <v>5400</v>
+        <v>586.32478632478603</v>
       </c>
       <c r="B192" s="1">
-        <v>46.153846153846096</v>
+        <v>25.274725274725199</v>
       </c>
       <c r="C192" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A193" s="1">
-        <v>5974.3589743589673</v>
+        <v>5386.3247863247798</v>
       </c>
       <c r="B193" s="1">
-        <v>60.439560439560402</v>
+        <v>27.4725274725274</v>
       </c>
       <c r="C193" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A194" s="1">
-        <v>6603.4188034187964</v>
+        <v>7109.4017094016999</v>
       </c>
       <c r="B194" s="1">
-        <v>76.923076923076906</v>
+        <v>62.087912087912002</v>
       </c>
       <c r="C194" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A195" s="1">
-        <v>6835.897435897431</v>
+        <v>7547.0085470085396</v>
       </c>
       <c r="B195" s="1">
-        <v>90.6593406593406</v>
+        <v>96.703296703296701</v>
       </c>
       <c r="C195" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A196" s="1">
-        <v>7013.6752136752148</v>
+        <v>6917.9487179487096</v>
       </c>
       <c r="B196" s="1">
-        <v>120.87912087911999</v>
+        <v>179.12087912087901</v>
       </c>
       <c r="C196" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A197" s="1">
-        <v>6781.1965811965783</v>
+        <v>6152.1367521367501</v>
       </c>
       <c r="B197" s="1">
-        <v>152.74725274725199</v>
+        <v>197.25274725274701</v>
       </c>
       <c r="C197" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A198" s="1">
-        <v>6343.5897435897432</v>
+        <v>4962.3931623931603</v>
       </c>
       <c r="B198" s="1">
-        <v>167.03296703296701</v>
+        <v>215.38461538461499</v>
       </c>
       <c r="C198" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A199" s="1">
-        <v>6015.3846153846107</v>
+        <v>3895.7264957264902</v>
       </c>
       <c r="B199" s="1">
-        <v>169.230769230769</v>
+        <v>225.274725274725</v>
       </c>
       <c r="C199" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A200" s="1">
-        <v>5755.5555555555484</v>
+        <v>-398.29059829059798</v>
       </c>
       <c r="B200" s="1">
-        <v>174.72527472527401</v>
+        <v>201.098901098901</v>
       </c>
       <c r="C200" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A201" s="1">
-        <v>4770.9401709401718</v>
+        <v>-1478.6324786324701</v>
       </c>
       <c r="B201" s="1">
-        <v>190.10989010988999</v>
+        <v>172.52747252747201</v>
       </c>
       <c r="C201" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A202" s="1">
-        <v>3964.1025641025599</v>
+        <v>-2217.0940170940098</v>
       </c>
       <c r="B202" s="1">
-        <v>200</v>
+        <v>139.56043956043899</v>
       </c>
       <c r="C202" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A203" s="1">
-        <v>3294.0170940170879</v>
+        <v>-2271.7948717948698</v>
       </c>
       <c r="B203" s="1">
-        <v>208.79120879120799</v>
+        <v>97.802197802197796</v>
       </c>
       <c r="C203" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A204" s="1">
-        <v>2487.1794871794846</v>
+        <v>-2011.96581196581</v>
       </c>
       <c r="B204" s="1">
-        <v>208.24175824175799</v>
+        <v>71.428571428571402</v>
       </c>
       <c r="C204" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A205" s="1">
-        <v>1694.0170940170908</v>
+        <v>-1464.9572649572599</v>
       </c>
       <c r="B205" s="1">
-        <v>201.648351648351</v>
+        <v>45.054945054945001</v>
       </c>
       <c r="C205" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A206" s="1">
-        <v>791.45299145299111</v>
+        <v>-740.17094017093996</v>
       </c>
       <c r="B206" s="1">
-        <v>190.10989010988999</v>
+        <v>30.769230769230699</v>
       </c>
       <c r="C206" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A207" s="1">
-        <v>449.57264957264988</v>
+        <v>2158.9743589743498</v>
       </c>
       <c r="B207" s="1">
-        <v>186.81318681318601</v>
+        <v>230.21978021978001</v>
       </c>
       <c r="C207" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A208" s="1">
-        <v>-439.31623931623858</v>
+        <v>859.82905982906004</v>
       </c>
       <c r="B208" s="1">
-        <v>171.97802197802099</v>
+        <v>215.93406593406499</v>
       </c>
       <c r="C208" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A209" s="1">
-        <v>-1314.5299145299111</v>
+        <v>1242.73504273504</v>
       </c>
       <c r="B209" s="1">
-        <v>149.450549450549</v>
+        <v>26.923076923076898</v>
       </c>
       <c r="C209" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A210" s="1">
-        <v>-1588.0341880341816</v>
+        <v>2705.9829059828999</v>
       </c>
       <c r="B210" s="1">
-        <v>126.373626373626</v>
+        <v>26.373626373626301</v>
       </c>
       <c r="C210" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A211" s="1">
-        <v>-1588.0341880341816</v>
+        <v>4155.5555555555502</v>
       </c>
       <c r="B211" s="1">
-        <v>92.307692307692193</v>
+        <v>26.373626373626301</v>
       </c>
       <c r="C211" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A212" s="1">
-        <v>-1423.9316239316158</v>
+        <v>6316.23931623931</v>
       </c>
       <c r="B212" s="1">
-        <v>76.923076923076906</v>
+        <v>37.912087912087898</v>
       </c>
       <c r="C212" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A213" s="1">
-        <v>-1068.3760683760668</v>
+        <v>7560.6837606837598</v>
       </c>
       <c r="B213" s="1">
-        <v>60.989010989011</v>
+        <v>136.81318681318601</v>
       </c>
       <c r="C213" s="1">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A214" s="1">
-        <v>-658.11965811965661</v>
+        <v>600</v>
       </c>
       <c r="B214" s="1">
-        <v>50.549450549450498</v>
+        <v>19.230769230769202</v>
       </c>
       <c r="C214" s="1">
-        <v>300</v>
+        <v>600</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A215" s="1">
-        <v>25.641025641026658</v>
+        <v>1967.5213675213599</v>
       </c>
       <c r="B215" s="1">
-        <v>39.560439560439498</v>
+        <v>19.230769230769202</v>
       </c>
       <c r="C215" s="1">
-        <v>300</v>
+        <v>600</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A216" s="1">
-        <v>572.64957264957263</v>
+        <v>3252.9914529914499</v>
       </c>
       <c r="B216" s="1">
-        <v>30.769230769230699</v>
+        <v>20.879120879120901</v>
       </c>
       <c r="C216" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A217" s="1">
-        <v>2528.2051282051289</v>
+        <v>5400</v>
       </c>
       <c r="B217" s="1">
-        <v>31.3186813186813</v>
+        <v>21.9780219780219</v>
       </c>
       <c r="C217" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A218" s="1">
-        <v>3280.3418803418795</v>
+        <v>6124.7863247863197</v>
       </c>
       <c r="B218" s="1">
-        <v>31.868131868131801</v>
+        <v>25.274725274725199</v>
       </c>
       <c r="C218" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A219" s="1">
-        <v>4511.1111111111095</v>
+        <v>7013.6752136752102</v>
       </c>
       <c r="B219" s="1">
-        <v>33.516483516483497</v>
+        <v>47.802197802197803</v>
       </c>
       <c r="C219" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A220" s="1">
-        <v>5400</v>
+        <v>7820.5128205128203</v>
       </c>
       <c r="B220" s="1">
-        <v>35.164835164835097</v>
+        <v>127.47252747252701</v>
       </c>
       <c r="C220" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A221" s="1">
-        <v>6070.0854700854634</v>
+        <v>7382.9059829059797</v>
       </c>
       <c r="B221" s="1">
-        <v>43.956043956043899</v>
+        <v>172.52747252747201</v>
       </c>
       <c r="C221" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A222" s="1">
-        <v>7041.0256410256407</v>
+        <v>6589.7435897435898</v>
       </c>
       <c r="B222" s="1">
-        <v>76.923076923076906</v>
+        <v>196.70329670329599</v>
       </c>
       <c r="C222" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A223" s="1">
-        <v>7410.2564102564074</v>
+        <v>5714.5299145299095</v>
       </c>
       <c r="B223" s="1">
-        <v>121.428571428571</v>
+        <v>215.38461538461499</v>
       </c>
       <c r="C223" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A224" s="1">
-        <v>6972.6495726495705</v>
+        <v>4729.9145299145202</v>
       </c>
       <c r="B224" s="1">
-        <v>160.43956043956001</v>
+        <v>227.47252747252699</v>
       </c>
       <c r="C224" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A225" s="1">
-        <v>6261.5384615384546</v>
+        <v>3649.5726495726499</v>
       </c>
       <c r="B225" s="1">
-        <v>180.21978021978001</v>
+        <v>236.26373626373601</v>
       </c>
       <c r="C225" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A226" s="1">
-        <v>4866.666666666667</v>
+        <v>2213.6752136752102</v>
       </c>
       <c r="B226" s="1">
-        <v>202.74725274725199</v>
+        <v>237.912087912087</v>
       </c>
       <c r="C226" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A227" s="1">
-        <v>3430.7692307692273</v>
+        <v>1174.35897435897</v>
       </c>
       <c r="B227" s="1">
-        <v>219.780219780219</v>
+        <v>224.72527472527401</v>
       </c>
       <c r="C227" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A228" s="1">
-        <v>2282.0512820512754</v>
+        <v>-193.16239316239299</v>
       </c>
       <c r="B228" s="1">
-        <v>219.780219780219</v>
+        <v>212.087912087912</v>
       </c>
       <c r="C228" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A229" s="1">
-        <v>1174.3589743589741</v>
+        <v>-1232.4786324786301</v>
       </c>
       <c r="B229" s="1">
-        <v>206.593406593406</v>
+        <v>190.65934065933999</v>
       </c>
       <c r="C229" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A230" s="1">
-        <v>-179.48717948717933</v>
+        <v>-2025.64102564102</v>
       </c>
       <c r="B230" s="1">
-        <v>189.01098901098899</v>
+        <v>167.03296703296701</v>
       </c>
       <c r="C230" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A231" s="1">
-        <v>-1068.3760683760668</v>
+        <v>-2435.8974358974301</v>
       </c>
       <c r="B231" s="1">
-        <v>170.32967032966999</v>
+        <v>139.01098901098899</v>
       </c>
       <c r="C231" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A232" s="1">
-        <v>-1683.7606837606777</v>
+        <v>-2545.29914529914</v>
       </c>
       <c r="B232" s="1">
-        <v>149.450549450549</v>
+        <v>109.890109890109</v>
       </c>
       <c r="C232" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A233" s="1">
-        <v>-1847.8632478632435</v>
+        <v>-2381.1965811965802</v>
       </c>
       <c r="B233" s="1">
-        <v>123.07692307692299</v>
+        <v>84.615384615384599</v>
       </c>
       <c r="C233" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A234" s="1">
-        <v>-1888.8888888888869</v>
+        <v>-1957.26495726495</v>
       </c>
       <c r="B234" s="1">
-        <v>93.956043956043899</v>
+        <v>56.593406593406598</v>
       </c>
       <c r="C234" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A235" s="1">
-        <v>-1560.6837606837553</v>
+        <v>-1492.3076923076901</v>
       </c>
       <c r="B235" s="1">
-        <v>67.582417582417506</v>
+        <v>38.461538461538403</v>
       </c>
       <c r="C235" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A236" s="1">
-        <v>-863.24786324785759</v>
+        <v>-781.19658119658095</v>
       </c>
       <c r="B236" s="1">
-        <v>42.857142857142797</v>
+        <v>24.1758241758242</v>
       </c>
       <c r="C236" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A237" s="1">
-        <v>-1.709401709401277</v>
+        <v>-206.83760683760599</v>
       </c>
       <c r="B237" s="1">
-        <v>31.3186813186813</v>
+        <v>19.230769230769202</v>
       </c>
       <c r="C237" s="1">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A238" s="1">
-        <v>586.32478632478694</v>
+        <v>4360.6837606837598</v>
       </c>
       <c r="B238" s="1">
-        <v>25.274725274725199</v>
+        <v>20.879120879120901</v>
       </c>
       <c r="C238" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A239" s="1">
-        <v>2022.2222222222226</v>
+        <v>7629.05982905983</v>
       </c>
       <c r="B239" s="1">
-        <v>25.274725274725199</v>
+        <v>86.263736263736206</v>
       </c>
       <c r="C239" s="1">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A240" s="1">
-        <v>3225.6410256410181</v>
+        <v>613.67521367521294</v>
       </c>
       <c r="B240" s="1">
-        <v>25.8241758241758</v>
+        <v>9.3406593406593199</v>
       </c>
       <c r="C240" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A241" s="1">
-        <v>5386.3247863247834</v>
+        <v>1844.44444444444</v>
       </c>
       <c r="B241" s="1">
-        <v>27.4725274725274</v>
+        <v>8.7912087912088097</v>
       </c>
       <c r="C241" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A242" s="1">
-        <v>5960.6837606837589</v>
+        <v>3266.6666666666601</v>
       </c>
       <c r="B242" s="1">
-        <v>29.6703296703296</v>
+        <v>9.8901098901098905</v>
       </c>
       <c r="C242" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A243" s="1">
-        <v>7109.4017094017099</v>
+        <v>5263.2478632478596</v>
       </c>
       <c r="B243" s="1">
-        <v>62.087912087912002</v>
+        <v>10.439560439560401</v>
       </c>
       <c r="C243" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A244" s="1">
-        <v>7547.0085470085478</v>
+        <v>6917.9487179487096</v>
       </c>
       <c r="B244" s="1">
-        <v>96.703296703296701</v>
+        <v>28.571428571428498</v>
       </c>
       <c r="C244" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A245" s="1">
-        <v>7683.7606837606781</v>
+        <v>7806.8376068376001</v>
       </c>
       <c r="B245" s="1">
-        <v>124.72527472527401</v>
+        <v>68.131868131868103</v>
       </c>
       <c r="C245" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A246" s="1">
-        <v>7437.6068376068333</v>
+        <v>8176.0683760683696</v>
       </c>
       <c r="B246" s="1">
-        <v>152.74725274725199</v>
+        <v>125.274725274725</v>
       </c>
       <c r="C246" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A247" s="1">
-        <v>6917.9487179487178</v>
+        <v>7875.2136752136703</v>
       </c>
       <c r="B247" s="1">
-        <v>179.12087912087901</v>
+        <v>168.681318681318</v>
       </c>
       <c r="C247" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A248" s="1">
-        <v>6152.1367521367501</v>
+        <v>7246.1538461538403</v>
       </c>
       <c r="B248" s="1">
-        <v>197.25274725274701</v>
+        <v>192.85714285714201</v>
       </c>
       <c r="C248" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A249" s="1">
-        <v>4962.3931623931549</v>
+        <v>5577.7777777777701</v>
       </c>
       <c r="B249" s="1">
-        <v>215.38461538461499</v>
+        <v>229.67032967032901</v>
       </c>
       <c r="C249" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A250" s="1">
-        <v>3895.7264957264902</v>
+        <v>4210.2564102564102</v>
       </c>
       <c r="B250" s="1">
-        <v>225.274725274725</v>
+        <v>241.75824175824101</v>
       </c>
       <c r="C250" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A251" s="1">
-        <v>2678.6324786324772</v>
+        <v>1680.3418803418799</v>
       </c>
       <c r="B251" s="1">
-        <v>229.67032967032901</v>
+        <v>240.65934065933999</v>
       </c>
       <c r="C251" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A252" s="1">
-        <v>1598.290598290595</v>
+        <v>217.094017094017</v>
       </c>
       <c r="B252" s="1">
-        <v>219.780219780219</v>
+        <v>226.923076923076</v>
       </c>
       <c r="C252" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A253" s="1">
-        <v>-398.29059829059486</v>
+        <v>-931.62393162393096</v>
       </c>
       <c r="B253" s="1">
-        <v>201.098901098901</v>
+        <v>210.98901098901001</v>
       </c>
       <c r="C253" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A254" s="1">
-        <v>-1478.6324786324772</v>
+        <v>-1533.3333333333301</v>
       </c>
       <c r="B254" s="1">
-        <v>172.52747252747201</v>
+        <v>195.60439560439499</v>
       </c>
       <c r="C254" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A255" s="1">
-        <v>-2217.0940170940103</v>
+        <v>-2353.8461538461502</v>
       </c>
       <c r="B255" s="1">
-        <v>139.56043956043899</v>
+        <v>170.32967032966999</v>
       </c>
       <c r="C255" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A256" s="1">
-        <v>-2271.7948717948716</v>
+        <v>-2695.7264957264902</v>
       </c>
       <c r="B256" s="1">
-        <v>97.802197802197796</v>
+        <v>138.461538461538</v>
       </c>
       <c r="C256" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A257" s="1">
-        <v>-2011.9658119658093</v>
+        <v>-2791.4529914529899</v>
       </c>
       <c r="B257" s="1">
-        <v>71.428571428571402</v>
+        <v>104.395604395604</v>
       </c>
       <c r="C257" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A258" s="1">
-        <v>-1464.9572649572597</v>
+        <v>-2572.64957264957</v>
       </c>
       <c r="B258" s="1">
-        <v>45.054945054945001</v>
+        <v>73.626373626373606</v>
       </c>
       <c r="C258" s="1">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="259" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A259" s="1">
-        <v>-740.17094017093541</v>
+        <v>-2107.6923076922999</v>
       </c>
       <c r="B259" s="1">
-        <v>30.769230769230699</v>
+        <v>45.604395604395499</v>
       </c>
       <c r="C259" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A260" s="1">
-        <v>189.74358974359069</v>
+        <v>-1615.38461538461</v>
       </c>
       <c r="B260" s="1">
-        <v>24.1758241758242</v>
+        <v>30.769230769230699</v>
       </c>
       <c r="C260" s="1">
-        <v>500</v>
+        <v>700</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A261" s="1">
-        <v>600</v>
+        <v>-917.94871794871699</v>
       </c>
       <c r="B261" s="1">
-        <v>19.230769230769202</v>
+        <v>14.8351648351648</v>
       </c>
       <c r="C261" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A262" s="1">
-        <v>1967.5213675213613</v>
+        <v>-111.11111111111001</v>
       </c>
       <c r="B262" s="1">
-        <v>19.230769230769202</v>
+        <v>9.8901098901098905</v>
       </c>
       <c r="C262" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A263" s="1">
-        <v>3252.9914529914445</v>
+        <v>6070.0854700854698</v>
       </c>
       <c r="B263" s="1">
-        <v>20.879120879120901</v>
+        <v>14.8351648351648</v>
       </c>
       <c r="C263" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A264" s="1">
-        <v>5400</v>
+        <v>4210.2564102564102</v>
       </c>
       <c r="B264" s="1">
-        <v>21.9780219780219</v>
+        <v>10.439560439560401</v>
       </c>
       <c r="C264" s="1">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A265" s="1">
-        <v>6124.7863247863243</v>
+        <v>586.32478632478603</v>
       </c>
       <c r="B265" s="1">
-        <v>25.274725274725199</v>
+        <v>0</v>
       </c>
       <c r="C265" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A266" s="1">
-        <v>7013.6752136752148</v>
+        <v>1762.3931623931601</v>
       </c>
       <c r="B266" s="1">
-        <v>47.802197802197803</v>
+        <v>0</v>
       </c>
       <c r="C266" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A267" s="1">
-        <v>7738.461538461539</v>
+        <v>3294.0170940170901</v>
       </c>
       <c r="B267" s="1">
-        <v>101.648351648351</v>
+        <v>0</v>
       </c>
       <c r="C267" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A268" s="1">
-        <v>7820.5128205128176</v>
+        <v>4675.2136752136703</v>
       </c>
       <c r="B268" s="1">
-        <v>127.47252747252701</v>
+        <v>0</v>
       </c>
       <c r="C268" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A269" s="1">
-        <v>7519.6581196581201</v>
+        <v>5441.0256410256397</v>
       </c>
       <c r="B269" s="1">
-        <v>157.142857142857</v>
+        <v>0</v>
       </c>
       <c r="C269" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A270" s="1">
-        <v>7382.9059829059806</v>
+        <v>6070.0854700854698</v>
       </c>
       <c r="B270" s="1">
-        <v>172.52747252747201</v>
+        <v>3.2967032967032899</v>
       </c>
       <c r="C270" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A271" s="1">
-        <v>6589.7435897435862</v>
+        <v>7205.1282051281996</v>
       </c>
       <c r="B271" s="1">
-        <v>196.70329670329599</v>
+        <v>15.934065934065901</v>
       </c>
       <c r="C271" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A272" s="1">
-        <v>5714.5299145299141</v>
+        <v>8203.4188034187991</v>
       </c>
       <c r="B272" s="1">
-        <v>215.38461538461499</v>
+        <v>70.329670329670293</v>
       </c>
       <c r="C272" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A273" s="1">
-        <v>4729.9145299145284</v>
+        <v>8176.0683760683696</v>
       </c>
       <c r="B273" s="1">
-        <v>227.47252747252699</v>
+        <v>160.43956043956001</v>
       </c>
       <c r="C273" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A274" s="1">
-        <v>3649.5726495726458</v>
+        <v>7341.88034188034</v>
       </c>
       <c r="B274" s="1">
-        <v>236.26373626373601</v>
+        <v>205.49450549450501</v>
       </c>
       <c r="C274" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A275" s="1">
-        <v>2801.7094017093991</v>
+        <v>6070.0854700854698</v>
       </c>
       <c r="B275" s="1">
-        <v>238.461538461538</v>
+        <v>236.26373626373601</v>
       </c>
       <c r="C275" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A276" s="1">
-        <v>2213.6752136752057</v>
+        <v>4264.9572649572601</v>
       </c>
       <c r="B276" s="1">
-        <v>237.912087912087</v>
+        <v>253.29670329670299</v>
       </c>
       <c r="C276" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A277" s="1">
-        <v>1174.3589743589741</v>
+        <v>1694.0170940170899</v>
       </c>
       <c r="B277" s="1">
-        <v>224.72527472527401</v>
+        <v>253.29670329670299</v>
       </c>
       <c r="C277" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A278" s="1">
-        <v>-193.16239316239239</v>
+        <v>162.39316239316199</v>
       </c>
       <c r="B278" s="1">
-        <v>212.087912087912</v>
+        <v>237.362637362637</v>
       </c>
       <c r="C278" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A279" s="1">
-        <v>-1232.4786324786241</v>
+        <v>-1054.70085470085</v>
       </c>
       <c r="B279" s="1">
-        <v>190.65934065933999</v>
+        <v>224.175824175824</v>
       </c>
       <c r="C279" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A280" s="1">
-        <v>-2025.6410256410181</v>
+        <v>-2135.0427350427299</v>
       </c>
       <c r="B280" s="1">
-        <v>167.03296703296701</v>
+        <v>194.505494505494</v>
       </c>
       <c r="C280" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A281" s="1">
-        <v>-2435.8974358974283</v>
+        <v>-2723.0769230769201</v>
       </c>
       <c r="B281" s="1">
-        <v>139.01098901098899</v>
+        <v>171.42857142857099</v>
       </c>
       <c r="C281" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A282" s="1">
-        <v>-2545.2991452991419</v>
+        <v>-2969.23076923076</v>
       </c>
       <c r="B282" s="1">
-        <v>109.890109890109</v>
+        <v>148.35164835164801</v>
       </c>
       <c r="C282" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A283" s="1">
-        <v>-2381.1965811965761</v>
+        <v>-2969.23076923076</v>
       </c>
       <c r="B283" s="1">
-        <v>84.615384615384599</v>
+        <v>84.065934065934002</v>
       </c>
       <c r="C283" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A284" s="1">
-        <v>-1957.264957264957</v>
+        <v>-2791.4529914529899</v>
       </c>
       <c r="B284" s="1">
-        <v>56.593406593406598</v>
+        <v>59.890109890109898</v>
       </c>
       <c r="C284" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A285" s="1">
-        <v>-1492.307692307686</v>
+        <v>-1943.58974358974</v>
       </c>
       <c r="B285" s="1">
-        <v>38.461538461538403</v>
+        <v>23.076923076922998</v>
       </c>
       <c r="C285" s="1">
-        <v>600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A286" s="1">
-        <v>-781.19658119657879</v>
+        <v>-658.11965811965797</v>
       </c>
       <c r="B286" s="1">
-        <v>24.1758241758242</v>
+        <v>1.6483516483516401</v>
       </c>
       <c r="C286" s="1">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A287" s="1">
-        <v>-206.83760683760647</v>
-      </c>
-      <c r="B287" s="1">
-        <v>19.230769230769202</v>
-      </c>
-      <c r="C287" s="1">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A288" s="1">
-        <v>613.67521367521385</v>
-      </c>
-      <c r="B288" s="1">
-        <v>9.3406593406593199</v>
-      </c>
-      <c r="C288" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A289" s="1">
-        <v>1270.0854700854693</v>
-      </c>
-      <c r="B289" s="1">
-        <v>9.8901098901098905</v>
-      </c>
-      <c r="C289" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A290" s="1">
-        <v>1434.1880341880344</v>
-      </c>
-      <c r="B290" s="1">
-        <v>7.6923076923076703</v>
-      </c>
-      <c r="C290" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A291" s="1">
-        <v>1844.4444444444393</v>
-      </c>
-      <c r="B291" s="1">
-        <v>8.7912087912088097</v>
-      </c>
-      <c r="C291" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A292" s="1">
-        <v>2637.6068376068333</v>
-      </c>
-      <c r="B292" s="1">
-        <v>9.8901098901098905</v>
-      </c>
-      <c r="C292" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A293" s="1">
-        <v>3266.6666666666615</v>
-      </c>
-      <c r="B293" s="1">
-        <v>9.8901098901098905</v>
-      </c>
-      <c r="C293" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A294" s="1">
-        <v>5263.2478632478606</v>
-      </c>
-      <c r="B294" s="1">
-        <v>10.439560439560401</v>
-      </c>
-      <c r="C294" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A295" s="1">
-        <v>5427.3504273504259</v>
-      </c>
-      <c r="B295" s="1">
-        <v>8.7912087912088097</v>
-      </c>
-      <c r="C295" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A296" s="1">
-        <v>5687.1794871794882</v>
-      </c>
-      <c r="B296" s="1">
-        <v>13.186813186813101</v>
-      </c>
-      <c r="C296" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A297" s="1">
-        <v>6917.9487179487178</v>
-      </c>
-      <c r="B297" s="1">
-        <v>28.571428571428498</v>
-      </c>
-      <c r="C297" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A298" s="1">
-        <v>7806.8376068376092</v>
-      </c>
-      <c r="B298" s="1">
-        <v>68.131868131868103</v>
-      </c>
-      <c r="C298" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A299" s="1">
-        <v>8094.0170940170865</v>
-      </c>
-      <c r="B299" s="1">
-        <v>101.098901098901</v>
-      </c>
-      <c r="C299" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A300" s="1">
-        <v>8176.0683760683751</v>
-      </c>
-      <c r="B300" s="1">
-        <v>125.274725274725</v>
-      </c>
-      <c r="C300" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A301" s="1">
-        <v>7984.615384615382</v>
-      </c>
-      <c r="B301" s="1">
-        <v>150.54945054945</v>
-      </c>
-      <c r="C301" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A302" s="1">
-        <v>7875.2136752136694</v>
-      </c>
-      <c r="B302" s="1">
-        <v>168.681318681318</v>
-      </c>
-      <c r="C302" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A303" s="1">
-        <v>7246.1538461538412</v>
-      </c>
-      <c r="B303" s="1">
-        <v>192.85714285714201</v>
-      </c>
-      <c r="C303" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A304" s="1">
-        <v>6562.3931623931603</v>
-      </c>
-      <c r="B304" s="1">
-        <v>208.24175824175799</v>
-      </c>
-      <c r="C304" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A305" s="1">
-        <v>5577.7777777777737</v>
-      </c>
-      <c r="B305" s="1">
-        <v>229.67032967032901</v>
-      </c>
-      <c r="C305" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A306" s="1">
-        <v>4880.3418803418763</v>
-      </c>
-      <c r="B306" s="1">
-        <v>236.26373626373601</v>
-      </c>
-      <c r="C306" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A307" s="1">
-        <v>4210.2564102564047</v>
-      </c>
-      <c r="B307" s="1">
-        <v>241.75824175824101</v>
-      </c>
-      <c r="C307" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A308" s="1">
-        <v>3471.7948717948716</v>
-      </c>
-      <c r="B308" s="1">
-        <v>247.25274725274701</v>
-      </c>
-      <c r="C308" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A309" s="1">
-        <v>2528.2051282051289</v>
-      </c>
-      <c r="B309" s="1">
-        <v>248.35164835164801</v>
-      </c>
-      <c r="C309" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A310" s="1">
-        <v>1680.3418803418733</v>
-      </c>
-      <c r="B310" s="1">
-        <v>240.65934065933999</v>
-      </c>
-      <c r="C310" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A311" s="1">
-        <v>217.09401709401772</v>
-      </c>
-      <c r="B311" s="1">
-        <v>226.923076923076</v>
-      </c>
-      <c r="C311" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A312" s="1">
-        <v>-931.62393162392732</v>
-      </c>
-      <c r="B312" s="1">
-        <v>210.98901098901001</v>
-      </c>
-      <c r="C312" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A313" s="1">
-        <v>-1533.3333333333294</v>
-      </c>
-      <c r="B313" s="1">
-        <v>195.60439560439499</v>
-      </c>
-      <c r="C313" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A314" s="1">
-        <v>-2353.8461538461502</v>
-      </c>
-      <c r="B314" s="1">
-        <v>170.32967032966999</v>
-      </c>
-      <c r="C314" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A315" s="1">
-        <v>-2695.7264957264902</v>
-      </c>
-      <c r="B315" s="1">
-        <v>138.461538461538</v>
-      </c>
-      <c r="C315" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A316" s="1">
-        <v>-2791.4529914529862</v>
-      </c>
-      <c r="B316" s="1">
-        <v>104.395604395604</v>
-      </c>
-      <c r="C316" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A317" s="1">
-        <v>-2572.6495726495677</v>
-      </c>
-      <c r="B317" s="1">
-        <v>73.626373626373606</v>
-      </c>
-      <c r="C317" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A318" s="1">
-        <v>-2107.6923076923053</v>
-      </c>
-      <c r="B318" s="1">
-        <v>45.604395604395499</v>
-      </c>
-      <c r="C318" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A319" s="1">
-        <v>-1615.384615384608</v>
-      </c>
-      <c r="B319" s="1">
-        <v>30.769230769230699</v>
-      </c>
-      <c r="C319" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A320" s="1">
-        <v>-917.9487179487096</v>
-      </c>
-      <c r="B320" s="1">
-        <v>14.8351648351648</v>
-      </c>
-      <c r="C320" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="321" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A321" s="1">
-        <v>-111.1111111111104</v>
-      </c>
-      <c r="B321" s="1">
-        <v>9.8901098901098905</v>
-      </c>
-      <c r="C321" s="1">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="322" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A322" s="1">
-        <v>586.32478632478694</v>
-      </c>
-      <c r="B322" s="1">
-        <v>0</v>
-      </c>
-      <c r="C322" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A323" s="1">
-        <v>1762.3931623931608</v>
-      </c>
-      <c r="B323" s="1">
-        <v>0</v>
-      </c>
-      <c r="C323" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="324" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A324" s="1">
-        <v>3294.0170940170879</v>
-      </c>
-      <c r="B324" s="1">
-        <v>0</v>
-      </c>
-      <c r="C324" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="325" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A325" s="1">
-        <v>4675.2136752136666</v>
-      </c>
-      <c r="B325" s="1">
-        <v>0</v>
-      </c>
-      <c r="C325" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="326" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A326" s="1">
-        <v>5441.0256410256343</v>
-      </c>
-      <c r="B326" s="1">
-        <v>0</v>
-      </c>
-      <c r="C326" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A327" s="1">
-        <v>6070.0854700854634</v>
-      </c>
-      <c r="B327" s="1">
-        <v>3.2967032967032899</v>
-      </c>
-      <c r="C327" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A328" s="1">
-        <v>6726.4957264957266</v>
-      </c>
-      <c r="B328" s="1">
-        <v>6.0439560439560296</v>
-      </c>
-      <c r="C328" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="329" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A329" s="1">
-        <v>7205.1282051282069</v>
-      </c>
-      <c r="B329" s="1">
-        <v>15.934065934065901</v>
-      </c>
-      <c r="C329" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="330" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A330" s="1">
-        <v>7765.8119658119649</v>
-      </c>
-      <c r="B330" s="1">
-        <v>39.010989010988901</v>
-      </c>
-      <c r="C330" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="331" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A331" s="1">
-        <v>8203.4188034188028</v>
-      </c>
-      <c r="B331" s="1">
-        <v>70.329670329670293</v>
-      </c>
-      <c r="C331" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="332" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A332" s="1">
-        <v>8176.0683760683751</v>
-      </c>
-      <c r="B332" s="1">
-        <v>160.43956043956001</v>
-      </c>
-      <c r="C332" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="333" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A333" s="1">
-        <v>7341.8803418803382</v>
-      </c>
-      <c r="B333" s="1">
-        <v>205.49450549450501</v>
-      </c>
-      <c r="C333" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="334" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A334" s="1">
-        <v>6070.0854700854634</v>
-      </c>
-      <c r="B334" s="1">
-        <v>236.26373626373601</v>
-      </c>
-      <c r="C334" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="335" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A335" s="1">
-        <v>4866.666666666667</v>
-      </c>
-      <c r="B335" s="1">
-        <v>249.450549450549</v>
-      </c>
-      <c r="C335" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="336" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A336" s="1">
-        <v>4264.9572649572656</v>
-      </c>
-      <c r="B336" s="1">
-        <v>253.29670329670299</v>
-      </c>
-      <c r="C336" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="337" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A337" s="1">
-        <v>1694.0170940170908</v>
-      </c>
-      <c r="B337" s="1">
-        <v>253.29670329670299</v>
-      </c>
-      <c r="C337" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="338" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A338" s="1">
-        <v>1037.6068376068372</v>
-      </c>
-      <c r="B338" s="1">
-        <v>247.80219780219701</v>
-      </c>
-      <c r="C338" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="339" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A339" s="1">
-        <v>162.39316239316275</v>
-      </c>
-      <c r="B339" s="1">
-        <v>237.362637362637</v>
-      </c>
-      <c r="C339" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="340" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A340" s="1">
-        <v>-576.06837606836962</v>
-      </c>
-      <c r="B340" s="1">
-        <v>231.868131868131</v>
-      </c>
-      <c r="C340" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="341" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A341" s="1">
-        <v>-1054.7008547008493</v>
-      </c>
-      <c r="B341" s="1">
-        <v>224.175824175824</v>
-      </c>
-      <c r="C341" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="342" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A342" s="1">
-        <v>-1629.0598290598255</v>
-      </c>
-      <c r="B342" s="1">
-        <v>210.98901098901001</v>
-      </c>
-      <c r="C342" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="343" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A343" s="1">
-        <v>-2135.0427350427317</v>
-      </c>
-      <c r="B343" s="1">
-        <v>194.505494505494</v>
-      </c>
-      <c r="C343" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="344" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A344" s="1">
-        <v>-2723.0769230769165</v>
-      </c>
-      <c r="B344" s="1">
-        <v>171.42857142857099</v>
-      </c>
-      <c r="C344" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="345" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A345" s="1">
-        <v>-2969.2307692307695</v>
-      </c>
-      <c r="B345" s="1">
-        <v>148.35164835164801</v>
-      </c>
-      <c r="C345" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="346" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A346" s="1">
-        <v>-2969.2307692307695</v>
-      </c>
-      <c r="B346" s="1">
-        <v>84.065934065934002</v>
-      </c>
-      <c r="C346" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="347" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A347" s="1">
-        <v>-2791.4529914529862</v>
-      </c>
-      <c r="B347" s="1">
-        <v>59.890109890109898</v>
-      </c>
-      <c r="C347" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="348" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A348" s="1">
-        <v>-2435.8974358974283</v>
-      </c>
-      <c r="B348" s="1">
-        <v>40.109890109890102</v>
-      </c>
-      <c r="C348" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="349" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A349" s="1">
-        <v>-1943.5897435897396</v>
-      </c>
-      <c r="B349" s="1">
-        <v>23.076923076922998</v>
-      </c>
-      <c r="C349" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="350" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A350" s="1">
-        <v>-1396.5811965811897</v>
-      </c>
-      <c r="B350" s="1">
-        <v>10.439560439560401</v>
-      </c>
-      <c r="C350" s="1">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="351" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A351" s="1">
-        <v>-658.11965811965661</v>
-      </c>
-      <c r="B351" s="1">
-        <v>1.6483516483516401</v>
-      </c>
-      <c r="C351" s="1">
         <v>800</v>
       </c>
     </row>

</xml_diff>